<commit_message>
Keep Excel answer validation compatible with the all-correct finale
</commit_message>
<xml_diff>
--- a/outputs/quiz-messi-20261006/Quiz-Messi-preguntas.xlsx
+++ b/outputs/quiz-messi-20261006/Quiz-Messi-preguntas.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preguntas" sheetId="1" r:id="R20e31a73651c4a2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preguntas" sheetId="1" r:id="R2697e1141b8f4e55"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5302,20 +5302,17 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="H8:H132">
-      <x:formula1>"A,B,C,D"</x:formula1>
-    </x:dataValidation>
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="J8:J132">
       <x:formula1>"Muy fácil,Fácil,Intermedio,Difícil,Experto"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="H132">
-      <x:formula1>"A,B,C,D,A, B, C y D"</x:formula1>
+    <x:dataValidation type="list" sqref="H8:H131">
+      <x:formula1>"A,B,C,D"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4482a7c5145e44e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4aff7dba58374a78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Open the quiz with Messi first Argentina shirt number
</commit_message>
<xml_diff>
--- a/outputs/quiz-messi-20261006/Quiz-Messi-preguntas.xlsx
+++ b/outputs/quiz-messi-20261006/Quiz-Messi-preguntas.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preguntas" sheetId="1" r:id="R2697e1141b8f4e55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preguntas" sheetId="1" r:id="Rdda0baaa4f114914"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -551,7 +551,7 @@
         <x:v>Fuente de revisión</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="62" customHeight="1">
+    <x:row r="8" ht="78" customHeight="1">
       <x:c r="A8" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -559,25 +559,25 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>¿Qué dos colores tiene la camiseta tradicional de Argentina?</x:v>
+        <x:v>¿Con qué número de camiseta debutó Messi con Argentina, en la Sub-20?</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>Verde y amarillo</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
-        <x:v>Azul y rojo</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
-        <x:v>Celeste y blanco</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G8" s="12" t="str">
-        <x:v>Rojo y blanco</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="H8" s="13" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I8" s="12" t="str">
-        <x:v>Messi defendió los colores celeste y blanco.</x:v>
+        <x:v>Messi debutó con la Sub-20 usando el 17, ante Paraguay el 29 de junio de 2004, en la cancha de Argentinos Juniors.</x:v>
       </x:c>
       <x:c r="J8" s="12" t="str">
         <x:v>Muy fácil</x:v>
@@ -586,7 +586,7 @@
         <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L8" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
+        <x:v>https://www.tycsports.com/seleccion-argentina/el-recuerdo-de-lionel-messi-a-20-anos-de-su-debut-con-la-seleccion-argentina-id593317.html</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="62" customHeight="1">
@@ -5312,7 +5312,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4aff7dba58374a78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3490ad5579b4247"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh quiz content, recover answers reliably and keep rankings current
</commit_message>
<xml_diff>
--- a/outputs/quiz-messi-20261006/Quiz-Messi-preguntas.xlsx
+++ b/outputs/quiz-messi-20261006/Quiz-Messi-preguntas.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preguntas" sheetId="1" r:id="Rdda0baaa4f114914"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preguntas" sheetId="1" r:id="R85d25757866546a0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -589,109 +589,109 @@
         <x:v>https://www.tycsports.com/seleccion-argentina/el-recuerdo-de-lionel-messi-a-20-anos-de-su-debut-con-la-seleccion-argentina-id593317.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="62" customHeight="1">
+    <x:row r="9" ht="110" customHeight="1">
       <x:c r="A9" s="8" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B9" s="8" t="n">
-        <x:v>67</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
-        <x:v>¿Qué apodo recibe la Selección Argentina por sus colores?</x:v>
+        <x:v>¿En qué estadio ganó Messi la Copa América 2021?</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>Centenario</x:v>
       </x:c>
       <x:c r="E9" s="12" t="str">
-        <x:v>La Azzurra</x:v>
+        <x:v>Maracaná</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
-        <x:v>La Canarinha</x:v>
+        <x:v>Wembley</x:v>
       </x:c>
       <x:c r="G9" s="12" t="str">
-        <x:v>La Roja</x:v>
+        <x:v>Monumental</x:v>
       </x:c>
       <x:c r="H9" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I9" s="12" t="str">
-        <x:v>El nombre remite al blanco y al celeste de su camiseta.</x:v>
+        <x:v>Argentina se consagró en el Maracaná de Río de Janeiro.</x:v>
       </x:c>
       <x:c r="J9" s="12" t="str">
         <x:v>Muy fácil</x:v>
       </x:c>
       <x:c r="K9" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L9" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="62" customHeight="1">
+    <x:row r="10" ht="110" customHeight="1">
       <x:c r="A10" s="8" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B10" s="8" t="n">
-        <x:v>55</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="C10" s="12" t="str">
-        <x:v>¿Qué número de camiseta identifica a Messi en la Selección desde 2009?</x:v>
+        <x:v>¿Quién hizo el único gol de la final de la Copa América 2021?</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>19</x:v>
+        <x:v>Ángel Di María</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
-        <x:v>10</x:v>
+        <x:v>Lautaro Martínez</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
-        <x:v>18</x:v>
+        <x:v>Sergio Agüero</x:v>
       </x:c>
       <x:c r="G10" s="12" t="str">
-        <x:v>7</x:v>
+        <x:v>Lionel Messi</x:v>
       </x:c>
       <x:c r="H10" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I10" s="12" t="str">
-        <x:v>El 10 es su número emblemático con Argentina.</x:v>
+        <x:v>Di María definió con un toque por encima de Ederson.</x:v>
       </x:c>
       <x:c r="J10" s="12" t="str">
         <x:v>Muy fácil</x:v>
       </x:c>
       <x:c r="K10" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L10" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="62" customHeight="1">
+    <x:row r="11" ht="110" customHeight="1">
       <x:c r="A11" s="8" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B11" s="8" t="n">
-        <x:v>88</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str">
-        <x:v>¿Quién dirigió a Messi en el Mundial de Qatar 2022?</x:v>
+        <x:v>¿Qué selección fue rival de Argentina en la final de Brasil 2014?</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
-        <x:v>Gerardo Martino</x:v>
+        <x:v>Francia</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
-        <x:v>Lionel Scaloni</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
-        <x:v>Jorge Sampaoli</x:v>
+        <x:v>Alemania</x:v>
       </x:c>
       <x:c r="G11" s="12" t="str">
-        <x:v>Alejandro Sabella</x:v>
+        <x:v>Países Bajos</x:v>
       </x:c>
       <x:c r="H11" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I11" s="12" t="str">
-        <x:v>Scaloni condujo al equipo campeón del mundo.</x:v>
+        <x:v>La final de 2014 enfrentó a Argentina y Alemania.</x:v>
       </x:c>
       <x:c r="J11" s="12" t="str">
         <x:v>Muy fácil</x:v>
@@ -703,71 +703,71 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="62" customHeight="1">
+    <x:row r="12" ht="110" customHeight="1">
       <x:c r="A12" s="8" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B12" s="8" t="n">
-        <x:v>96</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str">
-        <x:v>¿Contra qué selección ganó Messi la final de Qatar 2022?</x:v>
+        <x:v>¿Qué jugador terminó con más goles que Messi en Qatar 2022?</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>España</x:v>
+        <x:v>Julián Álvarez</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>Inglaterra</x:v>
+        <x:v>Harry Kane</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
-        <x:v>Alemania</x:v>
+        <x:v>Kylian Mbappé</x:v>
       </x:c>
       <x:c r="G12" s="12" t="str">
-        <x:v>Francia</x:v>
+        <x:v>Olivier Giroud</x:v>
       </x:c>
       <x:c r="H12" s="13" t="str">
-        <x:v>D</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I12" s="12" t="str">
-        <x:v>Argentina venció a Francia en una final inolvidable.</x:v>
+        <x:v>Mbappé marcó ocho goles y Messi, siete.</x:v>
       </x:c>
       <x:c r="J12" s="12" t="str">
         <x:v>Muy fácil</x:v>
       </x:c>
       <x:c r="K12" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>Qatar en detalle</x:v>
       </x:c>
       <x:c r="L12" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="62" customHeight="1">
+    <x:row r="13" ht="110" customHeight="1">
       <x:c r="A13" s="8" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="B13" s="8" t="n">
-        <x:v>100</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>¿En qué estadio levantó Messi la Copa del Mundo de 2022?</x:v>
+        <x:v>¿Qué selección venció a Argentina en su debut en Qatar 2022?</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>Wembley</x:v>
+        <x:v>Arabia Saudita</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
-        <x:v>Lusail</x:v>
+        <x:v>México</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
-        <x:v>Al Bayt</x:v>
+        <x:v>Polonia</x:v>
       </x:c>
       <x:c r="G13" s="12" t="str">
-        <x:v>Maracaná</x:v>
+        <x:v>Australia</x:v>
       </x:c>
       <x:c r="H13" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I13" s="12" t="str">
-        <x:v>La final se jugó en el Estadio de Lusail.</x:v>
+        <x:v>Argentina perdió 2-1 ante Arabia Saudita. Después ganó los seis cruces restantes, dos de ellos mediante tandas de penales.</x:v>
       </x:c>
       <x:c r="J13" s="12" t="str">
         <x:v>Muy fácil</x:v>
@@ -779,378 +779,378 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="62" customHeight="1">
+    <x:row r="14" ht="110" customHeight="1">
       <x:c r="A14" s="8" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="B14" s="8" t="n">
-        <x:v>113</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C14" s="12" t="str">
-        <x:v>¿En qué año ganó Messi su primera Copa América con la mayor?</x:v>
+        <x:v>¿Contra qué selección hizo Messi el primer gol del 2-0 que mantuvo vivo a Argentina en Qatar?</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>2021</x:v>
+        <x:v>Croacia</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
-        <x:v>2016</x:v>
+        <x:v>México</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
-        <x:v>2015</x:v>
+        <x:v>Australia</x:v>
       </x:c>
       <x:c r="G14" s="12" t="str">
-        <x:v>2019</x:v>
+        <x:v>Polonia</x:v>
       </x:c>
       <x:c r="H14" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I14" s="12" t="str">
-        <x:v>El primer título de Copa América de Leo llegó en 2021.</x:v>
+        <x:v>Su remate desde afuera del área abrió el partido ante México.</x:v>
       </x:c>
       <x:c r="J14" s="12" t="str">
         <x:v>Muy fácil</x:v>
       </x:c>
       <x:c r="K14" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L14" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="62" customHeight="1">
+    <x:row r="15" ht="110" customHeight="1">
       <x:c r="A15" s="8" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B15" s="8" t="n">
-        <x:v>114</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C15" s="12" t="str">
-        <x:v>¿A qué selección venció Argentina en la final de la Copa América 2021?</x:v>
+        <x:v>¿Quién pateó el penal que selló el título mundial de Messi en 2022?</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>Colombia</x:v>
+        <x:v>Paulo Dybala</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
-        <x:v>Uruguay</x:v>
+        <x:v>Leandro Paredes</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
-        <x:v>Chile</x:v>
+        <x:v>Lionel Messi</x:v>
       </x:c>
       <x:c r="G15" s="12" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Gonzalo Montiel</x:v>
       </x:c>
       <x:c r="H15" s="13" t="str">
         <x:v>D</x:v>
       </x:c>
       <x:c r="I15" s="12" t="str">
-        <x:v>Argentina venció 1-0 a Brasil.</x:v>
+        <x:v>Montiel convirtió el último penal de la final.</x:v>
       </x:c>
       <x:c r="J15" s="12" t="str">
         <x:v>Muy fácil</x:v>
       </x:c>
       <x:c r="K15" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>Qatar en detalle</x:v>
       </x:c>
       <x:c r="L15" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="62" customHeight="1">
+    <x:row r="16" ht="110" customHeight="1">
       <x:c r="A16" s="8" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B16" s="8" t="n">
-        <x:v>115</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C16" s="12" t="str">
-        <x:v>¿En qué estadio ganó Messi la Copa América 2021?</x:v>
+        <x:v>¿Qué selección fue rival de Messi en la semifinal de Qatar 2022?</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>Centenario</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>Maracaná</x:v>
+        <x:v>Portugal</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
-        <x:v>Wembley</x:v>
+        <x:v>Marruecos</x:v>
       </x:c>
       <x:c r="G16" s="12" t="str">
-        <x:v>Monumental</x:v>
+        <x:v>Croacia</x:v>
       </x:c>
       <x:c r="H16" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="I16" s="12" t="str">
-        <x:v>Argentina se consagró en el Maracaná de Río de Janeiro.</x:v>
+        <x:v>Argentina venció 3-0 a Croacia.</x:v>
       </x:c>
       <x:c r="J16" s="12" t="str">
         <x:v>Muy fácil</x:v>
       </x:c>
       <x:c r="K16" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L16" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="62" customHeight="1">
+    <x:row r="17" ht="110" customHeight="1">
       <x:c r="A17" s="8" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="B17" s="8" t="n">
-        <x:v>116</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C17" s="12" t="str">
-        <x:v>¿Quién hizo el único gol de la final de la Copa América 2021?</x:v>
+        <x:v>¿Cuántos goles con la mayor informa la AFA en el dato de referencia de esta edición?</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>Ángel Di María</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
-        <x:v>Lautaro Martínez</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="F17" s="12" t="str">
-        <x:v>Sergio Agüero</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="G17" s="12" t="str">
-        <x:v>Lionel Messi</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="H17" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I17" s="12" t="str">
-        <x:v>Di María definió con un toque por encima de Ederson.</x:v>
+        <x:v>La referencia fija de esta edición informa 125 goles de Messi con la Selección mayor. El banco contiene una pregunta por cada uno de esos goles.</x:v>
       </x:c>
       <x:c r="J17" s="12" t="str">
         <x:v>Muy fácil</x:v>
       </x:c>
       <x:c r="K17" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L17" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="62" customHeight="1">
+        <x:v>https://www.afa.com.ar/es/posts/125-goles-207-partidos-y-una-historia-que-cambio-para-siempre-a-la-seleccion-argentina</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="110" customHeight="1">
       <x:c r="A18" s="8" t="n">
         <x:v>11</x:v>
       </x:c>
       <x:c r="B18" s="8" t="n">
-        <x:v>81</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str">
-        <x:v>¿Qué selección fue rival de Argentina en la final de Brasil 2014?</x:v>
+        <x:v>¿En qué año Messi y todo el plantel argentino anunciaron que no hablarían más con la prensa?</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
-        <x:v>Francia</x:v>
+        <x:v>2014</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>2015</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
-        <x:v>Alemania</x:v>
+        <x:v>2016</x:v>
       </x:c>
       <x:c r="G18" s="12" t="str">
-        <x:v>Países Bajos</x:v>
+        <x:v>2018</x:v>
       </x:c>
       <x:c r="H18" s="13" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="I18" s="12" t="str">
-        <x:v>La final de 2014 enfrentó a Argentina y Alemania.</x:v>
+        <x:v>Fue el 15 de noviembre de 2016, después del 3-0 ante Colombia en San Juan. Messi anunció la decisión acompañado por sus compañeros, tras las acusaciones contra Ezequiel Lavezzi.</x:v>
       </x:c>
       <x:c r="J18" s="12" t="str">
-        <x:v>Muy fácil</x:v>
+        <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K18" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L18" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="62" customHeight="1">
+        <x:v>https://as.com/us/us/2016/11/16/futbol/1479272530_773720.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="110" customHeight="1">
       <x:c r="A19" s="8" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="B19" s="8" t="n">
-        <x:v>33</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="C19" s="12" t="str">
-        <x:v>¿Qué jugador terminó con más goles que Messi en Qatar 2022?</x:v>
+        <x:v>¿A qué jugador le dijo Messi «andá para allá, bobo» después del partido ante Países Bajos en Qatar 2022?</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
-        <x:v>Julián Álvarez</x:v>
+        <x:v>Wout Weghorst</x:v>
       </x:c>
       <x:c r="E19" s="12" t="str">
-        <x:v>Harry Kane</x:v>
+        <x:v>Denzel Dumfries</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
-        <x:v>Kylian Mbappé</x:v>
+        <x:v>Virgil van Dijk</x:v>
       </x:c>
       <x:c r="G19" s="12" t="str">
-        <x:v>Olivier Giroud</x:v>
+        <x:v>Memphis Depay</x:v>
       </x:c>
       <x:c r="H19" s="13" t="str">
-        <x:v>C</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I19" s="12" t="str">
-        <x:v>Mbappé marcó ocho goles y Messi, siete.</x:v>
+        <x:v>La frase estaba dirigida al delantero neerlandés Wout Weghorst, durante la entrevista con Gastón Edul después de los cuartos de final de Qatar 2022.</x:v>
       </x:c>
       <x:c r="J19" s="12" t="str">
-        <x:v>Muy fácil</x:v>
+        <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K19" s="12" t="str">
         <x:v>Qatar en detalle</x:v>
       </x:c>
       <x:c r="L19" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="62" customHeight="1">
+        <x:v>https://as.com/us/futbol/internacional/wout-weghorst-luego-de-que-messi-lo-llamo-bobo-al-menos-ya-sabe-mi-nombre-n/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="110" customHeight="1">
       <x:c r="A20" s="8" t="n">
         <x:v>13</x:v>
       </x:c>
       <x:c r="B20" s="8" t="n">
-        <x:v>89</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C20" s="12" t="str">
-        <x:v>¿Qué selección venció a Argentina en su debut en Qatar 2022?</x:v>
+        <x:v>¿Qué día nació Lionel Messi?</x:v>
       </x:c>
       <x:c r="D20" s="12" t="str">
-        <x:v>Arabia Saudita</x:v>
+        <x:v>24 de junio de 1987</x:v>
       </x:c>
       <x:c r="E20" s="12" t="str">
-        <x:v>México</x:v>
+        <x:v>24 de julio de 1987</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
-        <x:v>Polonia</x:v>
+        <x:v>21 de junio de 1987</x:v>
       </x:c>
       <x:c r="G20" s="12" t="str">
-        <x:v>Australia</x:v>
+        <x:v>24 de junio de 1986</x:v>
       </x:c>
       <x:c r="H20" s="13" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="I20" s="12" t="str">
-        <x:v>Argentina perdió 2-1 ante Arabia Saudita. Después ganó los seis cruces restantes, dos de ellos mediante tandas de penales.</x:v>
+        <x:v>Lionel Andrés Messi nació en Rosario, Santa Fe, el 24 de junio de 1987.</x:v>
       </x:c>
       <x:c r="J20" s="12" t="str">
-        <x:v>Muy fácil</x:v>
+        <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K20" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L20" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="62" customHeight="1">
+        <x:v>https://www.afa.com.ar/clubes/posts/lionel-messi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="110" customHeight="1">
       <x:c r="A21" s="8" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="B21" s="8" t="n">
-        <x:v>90</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C21" s="12" t="str">
-        <x:v>¿Contra qué selección hizo Messi el primer gol del 2-0 que mantuvo vivo a Argentina en Qatar?</x:v>
+        <x:v>¿En qué fecha ganó Messi la final del Mundial de Qatar 2022?</x:v>
       </x:c>
       <x:c r="D21" s="12" t="str">
-        <x:v>Croacia</x:v>
+        <x:v>20 de noviembre de 2022</x:v>
       </x:c>
       <x:c r="E21" s="12" t="str">
-        <x:v>México</x:v>
+        <x:v>10 de diciembre de 2022</x:v>
       </x:c>
       <x:c r="F21" s="12" t="str">
-        <x:v>Australia</x:v>
+        <x:v>18 de diciembre de 2022</x:v>
       </x:c>
       <x:c r="G21" s="12" t="str">
-        <x:v>Polonia</x:v>
+        <x:v>18 de noviembre de 2022</x:v>
       </x:c>
       <x:c r="H21" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I21" s="12" t="str">
-        <x:v>Su remate desde afuera del área abrió el partido ante México.</x:v>
+        <x:v>Argentina levantó la Copa el 18 de diciembre.</x:v>
       </x:c>
       <x:c r="J21" s="12" t="str">
-        <x:v>Muy fácil</x:v>
+        <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K21" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>Qatar en detalle</x:v>
       </x:c>
       <x:c r="L21" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="62" customHeight="1">
+    <x:row r="22" ht="110" customHeight="1">
       <x:c r="A22" s="8" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="B22" s="8" t="n">
-        <x:v>44</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C22" s="12" t="str">
-        <x:v>¿Quién pateó el penal que selló el título mundial de Messi en 2022?</x:v>
+        <x:v>¿Contra qué selección debutó Messi con la mayor en 2005?</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>Paulo Dybala</x:v>
+        <x:v>Croacia</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>Leandro Paredes</x:v>
+        <x:v>Paraguay</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
-        <x:v>Lionel Messi</x:v>
+        <x:v>Hungría</x:v>
       </x:c>
       <x:c r="G22" s="12" t="str">
-        <x:v>Gonzalo Montiel</x:v>
+        <x:v>Uruguay</x:v>
       </x:c>
       <x:c r="H22" s="13" t="str">
-        <x:v>D</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I22" s="12" t="str">
-        <x:v>Montiel convirtió el último penal de la final.</x:v>
+        <x:v>Su debut con la selección mayor fue ante Hungría.</x:v>
       </x:c>
       <x:c r="J22" s="12" t="str">
-        <x:v>Muy fácil</x:v>
+        <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K22" s="12" t="str">
-        <x:v>Qatar en detalle</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L22" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="62" customHeight="1">
+    <x:row r="23" ht="110" customHeight="1">
       <x:c r="A23" s="8" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="B23" s="8" t="n">
-        <x:v>94</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C23" s="12" t="str">
-        <x:v>¿Qué selección fue rival de Messi en la semifinal de Qatar 2022?</x:v>
+        <x:v>¿En qué país disputó Messi su primer Mundial de mayores?</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
+        <x:v>Sudáfrica</x:v>
+      </x:c>
+      <x:c r="E23" s="12" t="str">
+        <x:v>Francia</x:v>
+      </x:c>
+      <x:c r="F23" s="12" t="str">
         <x:v>Brasil</x:v>
       </x:c>
-      <x:c r="E23" s="12" t="str">
-        <x:v>Portugal</x:v>
-      </x:c>
-      <x:c r="F23" s="12" t="str">
-        <x:v>Marruecos</x:v>
-      </x:c>
       <x:c r="G23" s="12" t="str">
-        <x:v>Croacia</x:v>
+        <x:v>Alemania</x:v>
       </x:c>
       <x:c r="H23" s="13" t="str">
         <x:v>D</x:v>
       </x:c>
       <x:c r="I23" s="12" t="str">
-        <x:v>Argentina venció 3-0 a Croacia.</x:v>
+        <x:v>Su primera Copa del Mundo fue Alemania 2006.</x:v>
       </x:c>
       <x:c r="J23" s="12" t="str">
-        <x:v>Muy fácil</x:v>
+        <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K23" s="12" t="str">
         <x:v>Los Mundiales</x:v>
@@ -1159,36 +1159,36 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="62" customHeight="1">
+    <x:row r="24" ht="110" customHeight="1">
       <x:c r="A24" s="8" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="B24" s="8" t="n">
-        <x:v>45</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C24" s="12" t="str">
-        <x:v>¿Qué arquero argentino acompañó a Messi como titular durante Qatar 2022?</x:v>
+        <x:v>¿Qué edad tenía Messi al consagrarse campeón mundial en Qatar?</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>Emiliano Martínez</x:v>
+        <x:v>33 años</x:v>
       </x:c>
       <x:c r="E24" s="12" t="str">
-        <x:v>Gerónimo Rulli</x:v>
+        <x:v>35 años</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
-        <x:v>Franco Armani</x:v>
+        <x:v>36 años</x:v>
       </x:c>
       <x:c r="G24" s="12" t="str">
-        <x:v>Sergio Romero</x:v>
+        <x:v>34 años</x:v>
       </x:c>
       <x:c r="H24" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I24" s="12" t="str">
-        <x:v>Dibu Martínez defendió el arco durante los siete partidos.</x:v>
+        <x:v>Leo tenía 35 años cuando ganó la final.</x:v>
       </x:c>
       <x:c r="J24" s="12" t="str">
-        <x:v>Muy fácil</x:v>
+        <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K24" s="12" t="str">
         <x:v>Qatar en detalle</x:v>
@@ -1197,185 +1197,185 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="62" customHeight="1">
+    <x:row r="25" ht="110" customHeight="1">
       <x:c r="A25" s="8" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="B25" s="8" t="n">
-        <x:v>73</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C25" s="12" t="str">
-        <x:v>¿Cuántos goles con la mayor informa la AFA en el dato de referencia de esta edición?</x:v>
+        <x:v>¿Qué le ocurrió a Messi pocos segundos después de entrar en su debut con Argentina?</x:v>
       </x:c>
       <x:c r="D25" s="12" t="str">
-        <x:v>100</x:v>
+        <x:v>Fue capitán</x:v>
       </x:c>
       <x:c r="E25" s="12" t="str">
-        <x:v>125</x:v>
+        <x:v>Fue expulsado</x:v>
       </x:c>
       <x:c r="F25" s="12" t="str">
-        <x:v>115</x:v>
+        <x:v>Atajó un penal</x:v>
       </x:c>
       <x:c r="G25" s="12" t="str">
-        <x:v>130</x:v>
+        <x:v>Marcó dos goles</x:v>
       </x:c>
       <x:c r="H25" s="13" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="I25" s="12" t="str">
-        <x:v>La referencia fija de esta edición informa 125 goles de Messi con la Selección mayor. El banco contiene una pregunta por cada uno de esos goles.</x:v>
+        <x:v>Su estreno terminó con una expulsión.</x:v>
       </x:c>
       <x:c r="J25" s="12" t="str">
-        <x:v>Muy fácil</x:v>
+        <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K25" s="12" t="str">
         <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L25" s="11" t="str">
-        <x:v>https://www.afa.com.ar/es/posts/125-goles-207-partidos-y-una-historia-que-cambio-para-siempre-a-la-seleccion-argentina</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="62" customHeight="1">
+        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="110" customHeight="1">
       <x:c r="A26" s="8" t="n">
         <x:v>19</x:v>
       </x:c>
       <x:c r="B26" s="8" t="n">
-        <x:v>26</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C26" s="12" t="str">
-        <x:v>¿En qué fecha ganó Messi la final del Mundial de Qatar 2022?</x:v>
+        <x:v>¿En qué año debutó Messi con la Selección mayor?</x:v>
       </x:c>
       <x:c r="D26" s="12" t="str">
-        <x:v>20 de noviembre de 2022</x:v>
+        <x:v>2006</x:v>
       </x:c>
       <x:c r="E26" s="12" t="str">
-        <x:v>10 de diciembre de 2022</x:v>
+        <x:v>2004</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
-        <x:v>18 de diciembre de 2022</x:v>
+        <x:v>2007</x:v>
       </x:c>
       <x:c r="G26" s="12" t="str">
-        <x:v>18 de noviembre de 2022</x:v>
+        <x:v>2005</x:v>
       </x:c>
       <x:c r="H26" s="13" t="str">
-        <x:v>C</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="I26" s="12" t="str">
-        <x:v>Argentina levantó la Copa el 18 de diciembre.</x:v>
+        <x:v>Pekerman lo hizo debutar en agosto de 2005.</x:v>
       </x:c>
       <x:c r="J26" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K26" s="12" t="str">
-        <x:v>Qatar en detalle</x:v>
+        <x:v>El camino con Argentina</x:v>
       </x:c>
       <x:c r="L26" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="62" customHeight="1">
+    <x:row r="27" ht="110" customHeight="1">
       <x:c r="A27" s="8" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="B27" s="8" t="n">
-        <x:v>51</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="C27" s="12" t="str">
-        <x:v>¿Contra qué selección debutó Messi con la mayor en 2005?</x:v>
+        <x:v>¿Quién dirigió a Messi en el Mundial de Sudáfrica 2010?</x:v>
       </x:c>
       <x:c r="D27" s="12" t="str">
-        <x:v>Croacia</x:v>
+        <x:v>Alejandro Sabella</x:v>
       </x:c>
       <x:c r="E27" s="12" t="str">
-        <x:v>Paraguay</x:v>
+        <x:v>Jorge Sampaoli</x:v>
       </x:c>
       <x:c r="F27" s="12" t="str">
-        <x:v>Hungría</x:v>
+        <x:v>Diego Maradona</x:v>
       </x:c>
       <x:c r="G27" s="12" t="str">
-        <x:v>Uruguay</x:v>
+        <x:v>José Pekerman</x:v>
       </x:c>
       <x:c r="H27" s="13" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="I27" s="12" t="str">
-        <x:v>Su debut con la selección mayor fue ante Hungría.</x:v>
+        <x:v>Maradona fue el técnico argentino en 2010.</x:v>
       </x:c>
       <x:c r="J27" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K27" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L27" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="62" customHeight="1">
+    <x:row r="28" ht="110" customHeight="1">
       <x:c r="A28" s="8" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="B28" s="8" t="n">
-        <x:v>76</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C28" s="12" t="str">
-        <x:v>¿En qué país disputó Messi su primer Mundial de mayores?</x:v>
+        <x:v>¿En qué ciudad ganó Messi la medalla de oro olímpica en 2008?</x:v>
       </x:c>
       <x:c r="D28" s="12" t="str">
-        <x:v>Sudáfrica</x:v>
+        <x:v>Pekín</x:v>
       </x:c>
       <x:c r="E28" s="12" t="str">
-        <x:v>Francia</x:v>
+        <x:v>Río de Janeiro</x:v>
       </x:c>
       <x:c r="F28" s="12" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Londres</x:v>
       </x:c>
       <x:c r="G28" s="12" t="str">
-        <x:v>Alemania</x:v>
+        <x:v>Atenas</x:v>
       </x:c>
       <x:c r="H28" s="13" t="str">
-        <x:v>D</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I28" s="12" t="str">
-        <x:v>Su primera Copa del Mundo fue Alemania 2006.</x:v>
+        <x:v>Argentina fue campeona olímpica en Pekín 2008.</x:v>
       </x:c>
       <x:c r="J28" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K28" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L28" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="62" customHeight="1">
+    <x:row r="29" ht="110" customHeight="1">
       <x:c r="A29" s="8" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="B29" s="8" t="n">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str">
-        <x:v>¿Qué edad tenía Messi al consagrarse campeón mundial en Qatar?</x:v>
+        <x:v>¿Qué premio al mejor jugador recibió Messi en Qatar 2022?</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
-        <x:v>33 años</x:v>
+        <x:v>Balón de Oro del Mundial</x:v>
       </x:c>
       <x:c r="E29" s="12" t="str">
-        <x:v>35 años</x:v>
+        <x:v>Guante de Oro</x:v>
       </x:c>
       <x:c r="F29" s="12" t="str">
-        <x:v>36 años</x:v>
+        <x:v>Premio al mejor juvenil</x:v>
       </x:c>
       <x:c r="G29" s="12" t="str">
-        <x:v>34 años</x:v>
+        <x:v>Bota de Oro</x:v>
       </x:c>
       <x:c r="H29" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I29" s="12" t="str">
-        <x:v>Leo tenía 35 años cuando ganó la final.</x:v>
+        <x:v>La FIFA lo distinguió como mejor jugador del torneo.</x:v>
       </x:c>
       <x:c r="J29" s="12" t="str">
         <x:v>Fácil</x:v>
@@ -1387,33 +1387,33 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="62" customHeight="1">
+    <x:row r="30" ht="110" customHeight="1">
       <x:c r="A30" s="8" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="B30" s="8" t="n">
-        <x:v>52</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str">
-        <x:v>¿Qué le ocurrió a Messi pocos segundos después de entrar en su debut con Argentina?</x:v>
+        <x:v>¿Qué selección recibió cinco goles de Messi en un amistoso de 2022?</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>Fue capitán</x:v>
+        <x:v>Islandia</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>Fue expulsado</x:v>
+        <x:v>Lituania</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
-        <x:v>Atajó un penal</x:v>
+        <x:v>Letonia</x:v>
       </x:c>
       <x:c r="G30" s="12" t="str">
-        <x:v>Marcó dos goles</x:v>
+        <x:v>Estonia</x:v>
       </x:c>
       <x:c r="H30" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="I30" s="12" t="str">
-        <x:v>Su estreno terminó con una expulsión.</x:v>
+        <x:v>Messi convirtió los cinco goles del 5-0 a Estonia.</x:v>
       </x:c>
       <x:c r="J30" s="12" t="str">
         <x:v>Fácil</x:v>
@@ -1425,109 +1425,109 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="62" customHeight="1">
+    <x:row r="31" ht="110" customHeight="1">
       <x:c r="A31" s="8" t="n">
         <x:v>24</x:v>
       </x:c>
       <x:c r="B31" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C31" s="12" t="str">
-        <x:v>¿En qué año debutó Messi con la Selección mayor?</x:v>
+        <x:v>¿Qué selección venció a Argentina en la final de la Copa América 2007?</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>2006</x:v>
+        <x:v>Uruguay</x:v>
       </x:c>
       <x:c r="E31" s="12" t="str">
-        <x:v>2004</x:v>
+        <x:v>Chile</x:v>
       </x:c>
       <x:c r="F31" s="12" t="str">
-        <x:v>2007</x:v>
+        <x:v>Colombia</x:v>
       </x:c>
       <x:c r="G31" s="12" t="str">
-        <x:v>2005</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="H31" s="13" t="str">
         <x:v>D</x:v>
       </x:c>
       <x:c r="I31" s="12" t="str">
-        <x:v>Pekerman lo hizo debutar en agosto de 2005.</x:v>
+        <x:v>Brasil ganó la final de Venezuela 2007.</x:v>
       </x:c>
       <x:c r="J31" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K31" s="12" t="str">
-        <x:v>El camino con Argentina</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L31" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="62" customHeight="1">
+    <x:row r="32" ht="110" customHeight="1">
       <x:c r="A32" s="8" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="B32" s="8" t="n">
-        <x:v>79</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C32" s="12" t="str">
-        <x:v>¿Quién dirigió a Messi en el Mundial de Sudáfrica 2010?</x:v>
+        <x:v>¿Contra quién marcó Messi tres goles para clasificar a Rusia 2018?</x:v>
       </x:c>
       <x:c r="D32" s="12" t="str">
-        <x:v>Alejandro Sabella</x:v>
+        <x:v>Chile</x:v>
       </x:c>
       <x:c r="E32" s="12" t="str">
-        <x:v>Jorge Sampaoli</x:v>
+        <x:v>Ecuador</x:v>
       </x:c>
       <x:c r="F32" s="12" t="str">
-        <x:v>Diego Maradona</x:v>
+        <x:v>Colombia</x:v>
       </x:c>
       <x:c r="G32" s="12" t="str">
-        <x:v>José Pekerman</x:v>
+        <x:v>Perú</x:v>
       </x:c>
       <x:c r="H32" s="13" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I32" s="12" t="str">
-        <x:v>Maradona fue el técnico argentino en 2010.</x:v>
+        <x:v>Su hat-trick ante Ecuador aseguró la clasificación.</x:v>
       </x:c>
       <x:c r="J32" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K32" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L32" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="62" customHeight="1">
+    <x:row r="33" ht="110" customHeight="1">
       <x:c r="A33" s="8" t="n">
         <x:v>26</x:v>
       </x:c>
       <x:c r="B33" s="8" t="n">
-        <x:v>105</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="C33" s="12" t="str">
-        <x:v>¿En qué ciudad ganó Messi la medalla de oro olímpica en 2008?</x:v>
+        <x:v>¿Cuál es la famosa frase que dijo Messi después de perder la final de la Copa América 2016?</x:v>
       </x:c>
       <x:c r="D33" s="12" t="str">
-        <x:v>Pekín</x:v>
+        <x:v>Todavía queda una final por jugar.</x:v>
       </x:c>
       <x:c r="E33" s="12" t="str">
-        <x:v>Río de Janeiro</x:v>
+        <x:v>Es increíble pero no se me da.</x:v>
       </x:c>
       <x:c r="F33" s="12" t="str">
-        <x:v>Londres</x:v>
+        <x:v>No te largués, estamos viendo el partido.</x:v>
       </x:c>
       <x:c r="G33" s="12" t="str">
-        <x:v>Atenas</x:v>
+        <x:v>Nunca perdimos una final.</x:v>
       </x:c>
       <x:c r="H33" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I33" s="12" t="str">
-        <x:v>Argentina fue campeona olímpica en Pekín 2008.</x:v>
+        <x:v>Tras perder por penales ante Chile en 2016, Messi expresó su frustración: «Es increíble, pero no se me da». Luego regresó a la Selección.</x:v>
       </x:c>
       <x:c r="J33" s="12" t="str">
         <x:v>Fácil</x:v>
@@ -1536,264 +1536,264 @@
         <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L33" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="62" customHeight="1">
+        <x:v>https://www.elgrafico.com.ar/articulo/lionel-messi/66114/lionel-messi-y-su-fallida-renuncia-a-la-seleccion-me-pone-feliz-haberme-arrepentido · https://www.tycsports.com/gaming/la-pregunta-de-messi-que-incomodo-a-davo-xeneize-id695919.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="110" customHeight="1">
       <x:c r="A34" s="8" t="n">
         <x:v>27</x:v>
       </x:c>
       <x:c r="B34" s="8" t="n">
-        <x:v>31</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="C34" s="12" t="str">
-        <x:v>¿Qué premio al mejor jugador recibió Messi en Qatar 2022?</x:v>
+        <x:v>¿A quién asistió Messi con un centro para el último gol argentino ante Francia en Rusia 2018?</x:v>
       </x:c>
       <x:c r="D34" s="12" t="str">
-        <x:v>Balón de Oro del Mundial</x:v>
+        <x:v>Ángel Di María</x:v>
       </x:c>
       <x:c r="E34" s="12" t="str">
-        <x:v>Guante de Oro</x:v>
+        <x:v>Éver Banega</x:v>
       </x:c>
       <x:c r="F34" s="12" t="str">
-        <x:v>Premio al mejor juvenil</x:v>
+        <x:v>Sergio Agüero</x:v>
       </x:c>
       <x:c r="G34" s="12" t="str">
-        <x:v>Bota de Oro</x:v>
+        <x:v>Marcos Rojo</x:v>
       </x:c>
       <x:c r="H34" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I34" s="12" t="str">
-        <x:v>La FIFA lo distinguió como mejor jugador del torneo.</x:v>
+        <x:v>Messi envió el centro que Agüero cabeceó para el 4-3 final. Francia eliminó a Argentina en octavos de Rusia 2018.</x:v>
       </x:c>
       <x:c r="J34" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K34" s="12" t="str">
-        <x:v>Qatar en detalle</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L34" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="62" customHeight="1">
+        <x:v>https://www.fifa.com/es/tournaments/mens/worldcup</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="110" customHeight="1">
       <x:c r="A35" s="8" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="B35" s="8" t="n">
-        <x:v>57</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C35" s="12" t="str">
-        <x:v>¿Qué selección recibió cinco goles de Messi en un amistoso de 2022?</x:v>
+        <x:v>¿Cómo marcó Messi el gol argentino ante Arabia Saudita en Qatar 2022?</x:v>
       </x:c>
       <x:c r="D35" s="12" t="str">
-        <x:v>Islandia</x:v>
+        <x:v>De tiro libre</x:v>
       </x:c>
       <x:c r="E35" s="12" t="str">
-        <x:v>Lituania</x:v>
+        <x:v>De cabeza</x:v>
       </x:c>
       <x:c r="F35" s="12" t="str">
-        <x:v>Letonia</x:v>
+        <x:v>De chilena</x:v>
       </x:c>
       <x:c r="G35" s="12" t="str">
-        <x:v>Estonia</x:v>
+        <x:v>De penal</x:v>
       </x:c>
       <x:c r="H35" s="13" t="str">
         <x:v>D</x:v>
       </x:c>
       <x:c r="I35" s="12" t="str">
-        <x:v>Messi convirtió los cinco goles del 5-0 a Estonia.</x:v>
+        <x:v>Abrió el marcador desde el punto penal.</x:v>
       </x:c>
       <x:c r="J35" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K35" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>Qatar en detalle</x:v>
       </x:c>
       <x:c r="L35" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="62" customHeight="1">
+    <x:row r="36" ht="110" customHeight="1">
       <x:c r="A36" s="8" t="n">
         <x:v>29</x:v>
       </x:c>
       <x:c r="B36" s="8" t="n">
-        <x:v>108</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C36" s="12" t="str">
-        <x:v>¿Qué selección venció a Argentina en la final de la Copa América 2007?</x:v>
+        <x:v>¿Cómo terminó el partido de Argentina contra Suiza en octavos de Brasil 2014?</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
-        <x:v>Uruguay</x:v>
+        <x:v>Argentina ganó 1-0</x:v>
       </x:c>
       <x:c r="E36" s="12" t="str">
-        <x:v>Chile</x:v>
+        <x:v>Suiza ganó 2-1</x:v>
       </x:c>
       <x:c r="F36" s="12" t="str">
-        <x:v>Colombia</x:v>
+        <x:v>Argentina ganó 2-1</x:v>
       </x:c>
       <x:c r="G36" s="12" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Argentina ganó 2-0</x:v>
       </x:c>
       <x:c r="H36" s="13" t="str">
-        <x:v>D</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I36" s="12" t="str">
-        <x:v>Brasil ganó la final de Venezuela 2007.</x:v>
+        <x:v>Argentina ganó 1-0 en el alargue. Di María convirtió a los 118 minutos tras una asistencia de Messi.</x:v>
       </x:c>
       <x:c r="J36" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K36" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L36" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="62" customHeight="1">
+        <x:v>https://www.fifa.com/es/tournaments/mens/worldcup</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="110" customHeight="1">
       <x:c r="A37" s="8" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="B37" s="8" t="n">
-        <x:v>59</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C37" s="12" t="str">
-        <x:v>¿Contra quién marcó Messi tres goles para clasificar a Rusia 2018?</x:v>
+        <x:v>¿Cómo terminó el partido de octavos ante Australia, en el que Messi abrió el marcador?</x:v>
       </x:c>
       <x:c r="D37" s="12" t="str">
-        <x:v>Chile</x:v>
+        <x:v>Argentina ganó 1-0</x:v>
       </x:c>
       <x:c r="E37" s="12" t="str">
-        <x:v>Ecuador</x:v>
+        <x:v>Empataron 1-1</x:v>
       </x:c>
       <x:c r="F37" s="12" t="str">
-        <x:v>Colombia</x:v>
+        <x:v>Argentina ganó 3-0</x:v>
       </x:c>
       <x:c r="G37" s="12" t="str">
-        <x:v>Perú</x:v>
+        <x:v>Argentina ganó 2-1</x:v>
       </x:c>
       <x:c r="H37" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="I37" s="12" t="str">
-        <x:v>Su hat-trick ante Ecuador aseguró la clasificación.</x:v>
+        <x:v>Messi y Julián Álvarez anotaron para Argentina.</x:v>
       </x:c>
       <x:c r="J37" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K37" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>Qatar en detalle</x:v>
       </x:c>
       <x:c r="L37" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="78" customHeight="1">
+    <x:row r="38" ht="110" customHeight="1">
       <x:c r="A38" s="8" t="n">
         <x:v>31</x:v>
       </x:c>
       <x:c r="B38" s="8" t="n">
-        <x:v>109</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="C38" s="12" t="str">
-        <x:v>¿Cuál es la famosa frase que dijo Messi después de perder la final de la Copa América 2016?</x:v>
+        <x:v>¿Quién hizo el segundo gol argentino contra México en Qatar 2022?</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
-        <x:v>Todavía queda una final por jugar.</x:v>
+        <x:v>Enzo Fernández</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
-        <x:v>Es increíble pero no se me da.</x:v>
+        <x:v>Julián Álvarez</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
-        <x:v>Hoy ganamos la Copa América.</x:v>
+        <x:v>Lautaro Martínez</x:v>
       </x:c>
       <x:c r="G38" s="12" t="str">
-        <x:v>Nunca perdimos una final.</x:v>
+        <x:v>Ángel Di María</x:v>
       </x:c>
       <x:c r="H38" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I38" s="12" t="str">
-        <x:v>Tras perder por penales ante Chile en 2016, Messi expresó su frustración: «Es increíble, pero no se me da». Luego regresó a la Selección.</x:v>
+        <x:v>Enzo completó el 2-0 después del gol de Messi.</x:v>
       </x:c>
       <x:c r="J38" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K38" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L38" s="11" t="str">
-        <x:v>https://www.elgrafico.com.ar/articulo/lionel-messi/66114/lionel-messi-y-su-fallida-renuncia-a-la-seleccion-me-pone-feliz-haberme-arrepentido</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="62" customHeight="1">
+        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="110" customHeight="1">
       <x:c r="A39" s="8" t="n">
         <x:v>32</x:v>
       </x:c>
       <x:c r="B39" s="8" t="n">
-        <x:v>86</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C39" s="12" t="str">
-        <x:v>¿A quién asistió Messi con un centro para el último gol argentino ante Francia en Rusia 2018?</x:v>
+        <x:v>¿En qué instancia de la Copa América 2019 fue expulsado Messi ante Chile?</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>Ángel Di María</x:v>
+        <x:v>Semifinal</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
-        <x:v>Éver Banega</x:v>
+        <x:v>Cuartos de final</x:v>
       </x:c>
       <x:c r="F39" s="12" t="str">
-        <x:v>Sergio Agüero</x:v>
+        <x:v>Partido por el tercer puesto</x:v>
       </x:c>
       <x:c r="G39" s="12" t="str">
-        <x:v>Marcos Rojo</x:v>
+        <x:v>Final</x:v>
       </x:c>
       <x:c r="H39" s="13" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="I39" s="12" t="str">
-        <x:v>Messi envió el centro que Agüero cabeceó para el 4-3 final. Francia eliminó a Argentina en octavos de Rusia 2018.</x:v>
+        <x:v>Messi y Gary Medel fueron expulsados tras un cruce en el partido por el tercer puesto. Argentina venció 2-1 a Chile.</x:v>
       </x:c>
       <x:c r="J39" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K39" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>El camino con Argentina</x:v>
       </x:c>
       <x:c r="L39" s="11" t="str">
-        <x:v>https://www.fifa.com/es/tournaments/mens/worldcup</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="62" customHeight="1">
+        <x:v>https://cdn.conmebol.com/wp-content/uploads/2025/02/GET_CA_2019_ESP.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="110" customHeight="1">
       <x:c r="A40" s="8" t="n">
         <x:v>33</x:v>
       </x:c>
       <x:c r="B40" s="8" t="n">
-        <x:v>38</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="C40" s="12" t="str">
-        <x:v>¿Cómo marcó Messi el gol argentino ante Arabia Saudita en Qatar 2022?</x:v>
+        <x:v>¿Cómo terminó el partido contra Países Bajos en Qatar 2022 antes de la tanda?</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
-        <x:v>De tiro libre</x:v>
+        <x:v>1-1</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
-        <x:v>De cabeza</x:v>
+        <x:v>3-3</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
-        <x:v>De chilena</x:v>
+        <x:v>2-2</x:v>
       </x:c>
       <x:c r="G40" s="12" t="str">
-        <x:v>De penal</x:v>
+        <x:v>2-1 para Argentina</x:v>
       </x:c>
       <x:c r="H40" s="13" t="str">
-        <x:v>D</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I40" s="12" t="str">
-        <x:v>Abrió el marcador desde el punto penal.</x:v>
+        <x:v>Países Bajos igualó 2-2 y Argentina ganó por penales.</x:v>
       </x:c>
       <x:c r="J40" s="12" t="str">
         <x:v>Fácil</x:v>
@@ -1805,109 +1805,109 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="62" customHeight="1">
+    <x:row r="41" ht="110" customHeight="1">
       <x:c r="A41" s="8" t="n">
         <x:v>34</x:v>
       </x:c>
       <x:c r="B41" s="8" t="n">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C41" s="12" t="str">
-        <x:v>¿Cómo terminó el partido de Argentina contra Suiza en octavos de Brasil 2014?</x:v>
+        <x:v>¿Cuál fue el resultado de la tanda de penales en la final que ganó Messi en Qatar?</x:v>
       </x:c>
       <x:c r="D41" s="12" t="str">
-        <x:v>Argentina ganó 1-0</x:v>
+        <x:v>5-4 para Argentina</x:v>
       </x:c>
       <x:c r="E41" s="12" t="str">
-        <x:v>Suiza ganó 2-1</x:v>
+        <x:v>4-2 para Argentina</x:v>
       </x:c>
       <x:c r="F41" s="12" t="str">
-        <x:v>Argentina ganó 2-1</x:v>
+        <x:v>4-3 para Argentina</x:v>
       </x:c>
       <x:c r="G41" s="12" t="str">
-        <x:v>Argentina ganó 2-0</x:v>
+        <x:v>3-2 para Argentina</x:v>
       </x:c>
       <x:c r="H41" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I41" s="12" t="str">
-        <x:v>Argentina ganó 1-0 en el alargue. Di María convirtió a los 118 minutos tras una asistencia de Messi.</x:v>
+        <x:v>Argentina convirtió sus cuatro remates y Francia, dos.</x:v>
       </x:c>
       <x:c r="J41" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K41" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>Qatar en detalle</x:v>
       </x:c>
       <x:c r="L41" s="11" t="str">
-        <x:v>https://www.fifa.com/es/tournaments/mens/worldcup</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="62" customHeight="1">
+        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="110" customHeight="1">
       <x:c r="A42" s="8" t="n">
         <x:v>35</x:v>
       </x:c>
       <x:c r="B42" s="8" t="n">
-        <x:v>41</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C42" s="12" t="str">
-        <x:v>¿Cómo terminó el partido de octavos ante Australia, en el que Messi abrió el marcador?</x:v>
+        <x:v>¿Contra qué selección ganó Messi la Finalissima de 2022?</x:v>
       </x:c>
       <x:c r="D42" s="12" t="str">
-        <x:v>Argentina ganó 1-0</x:v>
+        <x:v>Francia</x:v>
       </x:c>
       <x:c r="E42" s="12" t="str">
-        <x:v>Empataron 1-1</x:v>
+        <x:v>Inglaterra</x:v>
       </x:c>
       <x:c r="F42" s="12" t="str">
-        <x:v>Argentina ganó 3-0</x:v>
+        <x:v>Portugal</x:v>
       </x:c>
       <x:c r="G42" s="12" t="str">
-        <x:v>Argentina ganó 2-1</x:v>
+        <x:v>Italia</x:v>
       </x:c>
       <x:c r="H42" s="13" t="str">
         <x:v>D</x:v>
       </x:c>
       <x:c r="I42" s="12" t="str">
-        <x:v>Messi y Julián Álvarez anotaron para Argentina.</x:v>
+        <x:v>Argentina venció 3-0 a Italia.</x:v>
       </x:c>
       <x:c r="J42" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K42" s="12" t="str">
-        <x:v>Qatar en detalle</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L42" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="62" customHeight="1">
+    <x:row r="43" ht="110" customHeight="1">
       <x:c r="A43" s="8" t="n">
         <x:v>36</x:v>
       </x:c>
       <x:c r="B43" s="8" t="n">
-        <x:v>91</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="C43" s="12" t="str">
-        <x:v>¿Quién hizo el segundo gol argentino contra México en Qatar 2022?</x:v>
+        <x:v>¿A qué delantero asistió Messi tras superar a Gvardiol en la semifinal de Qatar?</x:v>
       </x:c>
       <x:c r="D43" s="12" t="str">
-        <x:v>Enzo Fernández</x:v>
+        <x:v>Julián Álvarez</x:v>
       </x:c>
       <x:c r="E43" s="12" t="str">
-        <x:v>Julián Álvarez</x:v>
+        <x:v>Paulo Dybala</x:v>
       </x:c>
       <x:c r="F43" s="12" t="str">
         <x:v>Lautaro Martínez</x:v>
       </x:c>
       <x:c r="G43" s="12" t="str">
-        <x:v>Ángel Di María</x:v>
+        <x:v>Gonzalo Higuaín</x:v>
       </x:c>
       <x:c r="H43" s="13" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="I43" s="12" t="str">
-        <x:v>Enzo completó el 2-0 después del gol de Messi.</x:v>
+        <x:v>Julián convirtió el tercer gol ante Croacia.</x:v>
       </x:c>
       <x:c r="J43" s="12" t="str">
         <x:v>Fácil</x:v>
@@ -1919,71 +1919,71 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="62" customHeight="1">
+    <x:row r="44" ht="110" customHeight="1">
       <x:c r="A44" s="8" t="n">
         <x:v>37</x:v>
       </x:c>
       <x:c r="B44" s="8" t="n">
-        <x:v>17</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C44" s="12" t="str">
-        <x:v>¿En qué instancia de la Copa América 2019 fue expulsado Messi ante Chile?</x:v>
+        <x:v>¿En qué estadio ganó Messi la Finalissima 2022?</x:v>
       </x:c>
       <x:c r="D44" s="12" t="str">
-        <x:v>Semifinal</x:v>
+        <x:v>Maracaná</x:v>
       </x:c>
       <x:c r="E44" s="12" t="str">
-        <x:v>Cuartos de final</x:v>
+        <x:v>Wembley</x:v>
       </x:c>
       <x:c r="F44" s="12" t="str">
-        <x:v>Partido por el tercer puesto</x:v>
+        <x:v>San Siro</x:v>
       </x:c>
       <x:c r="G44" s="12" t="str">
-        <x:v>Final</x:v>
+        <x:v>Lusail</x:v>
       </x:c>
       <x:c r="H44" s="13" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I44" s="12" t="str">
-        <x:v>Messi y Gary Medel fueron expulsados tras un cruce en el partido por el tercer puesto. Argentina venció 2-1 a Chile.</x:v>
+        <x:v>La Finalissima se disputó en Wembley, Londres.</x:v>
       </x:c>
       <x:c r="J44" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K44" s="12" t="str">
-        <x:v>El camino con Argentina</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L44" s="11" t="str">
-        <x:v>https://cdn.conmebol.com/wp-content/uploads/2025/02/GET_CA_2019_ESP.pdf</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="62" customHeight="1">
+        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="110" customHeight="1">
       <x:c r="A45" s="8" t="n">
         <x:v>38</x:v>
       </x:c>
       <x:c r="B45" s="8" t="n">
-        <x:v>42</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C45" s="12" t="str">
-        <x:v>¿Cómo terminó el partido contra Países Bajos en Qatar 2022 antes de la tanda?</x:v>
+        <x:v>¿Qué arquero francés enfrentó Messi en la final de Qatar 2022?</x:v>
       </x:c>
       <x:c r="D45" s="12" t="str">
-        <x:v>1-1</x:v>
+        <x:v>Steve Mandanda</x:v>
       </x:c>
       <x:c r="E45" s="12" t="str">
-        <x:v>3-3</x:v>
+        <x:v>Alphonse Areola</x:v>
       </x:c>
       <x:c r="F45" s="12" t="str">
-        <x:v>2-2</x:v>
+        <x:v>Hugo Lloris</x:v>
       </x:c>
       <x:c r="G45" s="12" t="str">
-        <x:v>2-1 para Argentina</x:v>
+        <x:v>Mike Maignan</x:v>
       </x:c>
       <x:c r="H45" s="13" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="I45" s="12" t="str">
-        <x:v>Países Bajos igualó 2-2 y Argentina ganó por penales.</x:v>
+        <x:v>Lloris fue el arquero titular de Francia.</x:v>
       </x:c>
       <x:c r="J45" s="12" t="str">
         <x:v>Fácil</x:v>
@@ -1995,185 +1995,185 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="62" customHeight="1">
+    <x:row r="46" ht="110" customHeight="1">
       <x:c r="A46" s="8" t="n">
         <x:v>39</x:v>
       </x:c>
       <x:c r="B46" s="8" t="n">
-        <x:v>43</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="C46" s="12" t="str">
-        <x:v>¿Cuál fue el resultado de la tanda de penales en la final que ganó Messi en Qatar?</x:v>
+        <x:v>¿Qué selección fue rival de Argentina en la final de la Copa América 2024?</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
-        <x:v>5-4 para Argentina</x:v>
+        <x:v>Ecuador</x:v>
       </x:c>
       <x:c r="E46" s="12" t="str">
-        <x:v>4-2 para Argentina</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="F46" s="12" t="str">
-        <x:v>4-3 para Argentina</x:v>
+        <x:v>Uruguay</x:v>
       </x:c>
       <x:c r="G46" s="12" t="str">
-        <x:v>3-2 para Argentina</x:v>
+        <x:v>Colombia</x:v>
       </x:c>
       <x:c r="H46" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="I46" s="12" t="str">
-        <x:v>Argentina convirtió sus cuatro remates y Francia, dos.</x:v>
+        <x:v>Argentina venció a Colombia en el alargue.</x:v>
       </x:c>
       <x:c r="J46" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K46" s="12" t="str">
-        <x:v>Qatar en detalle</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L46" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="62" customHeight="1">
+    <x:row r="47" ht="110" customHeight="1">
       <x:c r="A47" s="8" t="n">
         <x:v>40</x:v>
       </x:c>
       <x:c r="B47" s="8" t="n">
-        <x:v>119</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="C47" s="12" t="str">
-        <x:v>¿Contra qué selección ganó Messi la Finalissima de 2022?</x:v>
+        <x:v>¿Cuántos goles hizo Messi durante el partido de la final de Qatar 2022, sin contar la tanda?</x:v>
       </x:c>
       <x:c r="D47" s="12" t="str">
-        <x:v>Francia</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E47" s="12" t="str">
-        <x:v>Inglaterra</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F47" s="12" t="str">
-        <x:v>Portugal</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G47" s="12" t="str">
-        <x:v>Italia</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H47" s="13" t="str">
         <x:v>D</x:v>
       </x:c>
       <x:c r="I47" s="12" t="str">
-        <x:v>Argentina venció 3-0 a Italia.</x:v>
+        <x:v>Marcó de penal y volvió a anotar en el alargue.</x:v>
       </x:c>
       <x:c r="J47" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K47" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L47" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="62" customHeight="1">
+    <x:row r="48" ht="110" customHeight="1">
       <x:c r="A48" s="8" t="n">
         <x:v>41</x:v>
       </x:c>
       <x:c r="B48" s="8" t="n">
-        <x:v>95</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="C48" s="12" t="str">
-        <x:v>¿A qué delantero asistió Messi tras superar a Gvardiol en la semifinal de Qatar?</x:v>
+        <x:v>¿Quién marcó el gol del título argentino en la Copa América 2024?</x:v>
       </x:c>
       <x:c r="D48" s="12" t="str">
         <x:v>Julián Álvarez</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
-        <x:v>Paulo Dybala</x:v>
+        <x:v>Lautaro Martínez</x:v>
       </x:c>
       <x:c r="F48" s="12" t="str">
-        <x:v>Lautaro Martínez</x:v>
+        <x:v>Lionel Messi</x:v>
       </x:c>
       <x:c r="G48" s="12" t="str">
-        <x:v>Gonzalo Higuaín</x:v>
+        <x:v>Ángel Di María</x:v>
       </x:c>
       <x:c r="H48" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I48" s="12" t="str">
-        <x:v>Julián convirtió el tercer gol ante Croacia.</x:v>
+        <x:v>Lautaro hizo el 1-0 definitivo.</x:v>
       </x:c>
       <x:c r="J48" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K48" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L48" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="62" customHeight="1">
+    <x:row r="49" ht="110" customHeight="1">
       <x:c r="A49" s="8" t="n">
         <x:v>42</x:v>
       </x:c>
       <x:c r="B49" s="8" t="n">
-        <x:v>120</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="C49" s="12" t="str">
-        <x:v>¿En qué estadio ganó Messi la Finalissima 2022?</x:v>
+        <x:v>¿Cuál fue el resultado de la final de Qatar 2022 antes de los penales?</x:v>
       </x:c>
       <x:c r="D49" s="12" t="str">
-        <x:v>Maracaná</x:v>
+        <x:v>3-3</x:v>
       </x:c>
       <x:c r="E49" s="12" t="str">
-        <x:v>Wembley</x:v>
+        <x:v>2-1</x:v>
       </x:c>
       <x:c r="F49" s="12" t="str">
-        <x:v>San Siro</x:v>
+        <x:v>2-2</x:v>
       </x:c>
       <x:c r="G49" s="12" t="str">
-        <x:v>Lusail</x:v>
+        <x:v>4-3</x:v>
       </x:c>
       <x:c r="H49" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I49" s="12" t="str">
-        <x:v>La Finalissima se disputó en Wembley, Londres.</x:v>
+        <x:v>Francia y Argentina empataron 3-3 tras el alargue.</x:v>
       </x:c>
       <x:c r="J49" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K49" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L49" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="62" customHeight="1">
+    <x:row r="50" ht="110" customHeight="1">
       <x:c r="A50" s="8" t="n">
         <x:v>43</x:v>
       </x:c>
       <x:c r="B50" s="8" t="n">
-        <x:v>46</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C50" s="12" t="str">
-        <x:v>¿Qué arquero francés enfrentó Messi en la final de Qatar 2022?</x:v>
+        <x:v>¿Qué árbitro cobró el penal que Messi convirtió ante Croacia en la semifinal de Qatar 2022?</x:v>
       </x:c>
       <x:c r="D50" s="12" t="str">
-        <x:v>Steve Mandanda</x:v>
+        <x:v>Mateu Lahoz</x:v>
       </x:c>
       <x:c r="E50" s="12" t="str">
-        <x:v>Alphonse Areola</x:v>
+        <x:v>Szymon Marciniak</x:v>
       </x:c>
       <x:c r="F50" s="12" t="str">
-        <x:v>Hugo Lloris</x:v>
+        <x:v>Daniele Orsato</x:v>
       </x:c>
       <x:c r="G50" s="12" t="str">
-        <x:v>Mike Maignan</x:v>
+        <x:v>Michael Oliver</x:v>
       </x:c>
       <x:c r="H50" s="13" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="I50" s="12" t="str">
-        <x:v>Lloris fue el arquero titular de Francia.</x:v>
+        <x:v>El italiano Daniele Orsato dirigió la semifinal del 13 de diciembre de 2022. Cobró el penal que Messi convirtió para abrir el 3-0 de Argentina ante Croacia.</x:v>
       </x:c>
       <x:c r="J50" s="12" t="str">
         <x:v>Fácil</x:v>
@@ -2182,229 +2182,229 @@
         <x:v>Qatar en detalle</x:v>
       </x:c>
       <x:c r="L50" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51" ht="62" customHeight="1">
+        <x:v>https://www.afa.com.ar/es/posts/sinstesis-mundial</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="110" customHeight="1">
       <x:c r="A51" s="8" t="n">
         <x:v>44</x:v>
       </x:c>
       <x:c r="B51" s="8" t="n">
-        <x:v>121</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="C51" s="12" t="str">
-        <x:v>¿Qué selección fue rival de Argentina en la final de la Copa América 2024?</x:v>
+        <x:v>¿Cuántos goles hizo Messi en todo el Mundial de Qatar 2022?</x:v>
       </x:c>
       <x:c r="D51" s="12" t="str">
-        <x:v>Ecuador</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E51" s="12" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F51" s="12" t="str">
-        <x:v>Uruguay</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G51" s="12" t="str">
-        <x:v>Colombia</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H51" s="13" t="str">
         <x:v>D</x:v>
       </x:c>
       <x:c r="I51" s="12" t="str">
-        <x:v>Argentina venció a Colombia en el alargue.</x:v>
+        <x:v>Leo terminó el torneo con siete goles.</x:v>
       </x:c>
       <x:c r="J51" s="12" t="str">
         <x:v>Fácil</x:v>
       </x:c>
       <x:c r="K51" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L51" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="62" customHeight="1">
+    <x:row r="52" ht="110" customHeight="1">
       <x:c r="A52" s="8" t="n">
         <x:v>45</x:v>
       </x:c>
       <x:c r="B52" s="8" t="n">
-        <x:v>97</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C52" s="12" t="str">
-        <x:v>¿Cuántos goles hizo Messi durante el partido de la final de Qatar 2022, sin contar la tanda?</x:v>
+        <x:v>¿Contra qué selección jugó Messi su partido número 200 con Argentina?</x:v>
       </x:c>
       <x:c r="D52" s="12" t="str">
-        <x:v>3</x:v>
+        <x:v>Argelia</x:v>
       </x:c>
       <x:c r="E52" s="12" t="str">
-        <x:v>0</x:v>
+        <x:v>Austria</x:v>
       </x:c>
       <x:c r="F52" s="12" t="str">
-        <x:v>1</x:v>
+        <x:v>Jordania</x:v>
       </x:c>
       <x:c r="G52" s="12" t="str">
-        <x:v>2</x:v>
+        <x:v>Egipto</x:v>
       </x:c>
       <x:c r="H52" s="13" t="str">
-        <x:v>D</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I52" s="12" t="str">
-        <x:v>Marcó de penal y volvió a anotar en el alargue.</x:v>
+        <x:v>Messi llegó a los 200 partidos con la Selección mayor ante Argelia, en el debut de Argentina en el Mundial 2026, el 16 de junio.</x:v>
       </x:c>
       <x:c r="J52" s="12" t="str">
-        <x:v>Fácil</x:v>
+        <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K52" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L52" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="62" customHeight="1">
+        <x:v>https://www.afa.com.ar/936/posts/messi-y-una-cifra-imposible-200-veces-argentina-200-veces-el-sueno-de-todos</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="110" customHeight="1">
       <x:c r="A53" s="8" t="n">
         <x:v>46</x:v>
       </x:c>
       <x:c r="B53" s="8" t="n">
-        <x:v>122</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C53" s="12" t="str">
-        <x:v>¿Quién marcó el gol del título argentino en la Copa América 2024?</x:v>
+        <x:v>¿Cuántos números de camiseta diferentes usó Messi con la Selección mayor?</x:v>
       </x:c>
       <x:c r="D53" s="12" t="str">
-        <x:v>Julián Álvarez</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E53" s="12" t="str">
-        <x:v>Lautaro Martínez</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F53" s="12" t="str">
-        <x:v>Lionel Messi</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G53" s="12" t="str">
-        <x:v>Ángel Di María</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H53" s="13" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="I53" s="12" t="str">
-        <x:v>Lautaro hizo el 1-0 definitivo.</x:v>
+        <x:v>Con la Selección mayor usó los dorsales 18, 19 y 10: tres números diferentes. No se cuentan la Sub-20 ni la selección olímpica, donde también llevó otros números.</x:v>
       </x:c>
       <x:c r="J53" s="12" t="str">
-        <x:v>Fácil</x:v>
+        <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K53" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L53" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54" ht="62" customHeight="1">
+        <x:v>https://www.elgrafico.com.ar/articulo/%C2%A1habla-memoria%21/35208/2010-messi-100x100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="110" customHeight="1">
       <x:c r="A54" s="8" t="n">
         <x:v>47</x:v>
       </x:c>
       <x:c r="B54" s="8" t="n">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C54" s="12" t="str">
-        <x:v>¿Cuál fue el resultado de la final de Qatar 2022 antes de los penales?</x:v>
+        <x:v>¿Contra qué selección hizo Messi su primer gol de tiro libre con Argentina?</x:v>
       </x:c>
       <x:c r="D54" s="12" t="str">
-        <x:v>3-3</x:v>
+        <x:v>Uruguay</x:v>
       </x:c>
       <x:c r="E54" s="12" t="str">
-        <x:v>2-1</x:v>
+        <x:v>Paraguay</x:v>
       </x:c>
       <x:c r="F54" s="12" t="str">
-        <x:v>2-2</x:v>
+        <x:v>Chile</x:v>
       </x:c>
       <x:c r="G54" s="12" t="str">
-        <x:v>4-3</x:v>
+        <x:v>Colombia</x:v>
       </x:c>
       <x:c r="H54" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I54" s="12" t="str">
-        <x:v>Francia y Argentina empataron 3-3 tras el alargue.</x:v>
+        <x:v>Fue ante Paraguay, el 7 de septiembre de 2012, en el estadio Mario Alberto Kempes de Córdoba. Messi marcó de tiro libre en el triunfo argentino por 3-1 por las Eliminatorias para Brasil 2014.</x:v>
       </x:c>
       <x:c r="J54" s="12" t="str">
-        <x:v>Fácil</x:v>
+        <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K54" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L54" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55" ht="62" customHeight="1">
+        <x:v>https://www.lanacion.com.ar/deportes/futbol/lionel-messi-su-conexion-paraguay-del-operativo-nid2506674/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="110" customHeight="1">
       <x:c r="A55" s="8" t="n">
         <x:v>48</x:v>
       </x:c>
       <x:c r="B55" s="8" t="n">
-        <x:v>49</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C55" s="12" t="str">
-        <x:v>¿Cuántos goles hizo Julián Álvarez junto a Messi en la semifinal ante Croacia?</x:v>
+        <x:v>¿A qué selección le hizo Messi el gol de tiro libre por abajo de la barrera en octubre de 2012?</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
-        <x:v>1</x:v>
+        <x:v>Paraguay</x:v>
       </x:c>
       <x:c r="E55" s="12" t="str">
-        <x:v>3</x:v>
+        <x:v>Ecuador</x:v>
       </x:c>
       <x:c r="F55" s="12" t="str">
-        <x:v>2</x:v>
+        <x:v>Uruguay</x:v>
       </x:c>
       <x:c r="G55" s="12" t="str">
-        <x:v>0</x:v>
+        <x:v>Bolivia</x:v>
       </x:c>
       <x:c r="H55" s="13" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="I55" s="12" t="str">
-        <x:v>Julián marcó dos goles y Messi uno en el 3-0.</x:v>
+        <x:v>Messi sorprendió a Uruguay con un remate rasante por debajo de la barrera, el 12 de octubre de 2012 en Mendoza. Fue el tercer gol del 3-0 argentino por las Eliminatorias para Brasil 2014.</x:v>
       </x:c>
       <x:c r="J55" s="12" t="str">
-        <x:v>Fácil</x:v>
+        <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K55" s="12" t="str">
-        <x:v>Qatar en detalle</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L55" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="62" customHeight="1">
+        <x:v>https://www.tycsports.com/futbol/el-dia-que-messi-engano-todo-uruguay.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="110" customHeight="1">
       <x:c r="A56" s="8" t="n">
         <x:v>49</x:v>
       </x:c>
       <x:c r="B56" s="8" t="n">
-        <x:v>99</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C56" s="12" t="str">
-        <x:v>¿Cuántos goles hizo Messi en todo el Mundial de Qatar 2022?</x:v>
+        <x:v>¿Contra qué selección marcó Messi su primer gol mundialista?</x:v>
       </x:c>
       <x:c r="D56" s="12" t="str">
-        <x:v>8</x:v>
+        <x:v>México</x:v>
       </x:c>
       <x:c r="E56" s="12" t="str">
-        <x:v>5</x:v>
+        <x:v>Costa de Marfil</x:v>
       </x:c>
       <x:c r="F56" s="12" t="str">
-        <x:v>6</x:v>
+        <x:v>Serbia y Montenegro</x:v>
       </x:c>
       <x:c r="G56" s="12" t="str">
-        <x:v>7</x:v>
+        <x:v>Países Bajos</x:v>
       </x:c>
       <x:c r="H56" s="13" t="str">
-        <x:v>D</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I56" s="12" t="str">
-        <x:v>Leo terminó el torneo con siete goles.</x:v>
+        <x:v>Marcó en el 6-0 de Argentina en 2006.</x:v>
       </x:c>
       <x:c r="J56" s="12" t="str">
-        <x:v>Fácil</x:v>
+        <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K56" s="12" t="str">
         <x:v>Los Mundiales</x:v>
@@ -2413,71 +2413,71 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="62" customHeight="1">
+    <x:row r="57" ht="110" customHeight="1">
       <x:c r="A57" s="8" t="n">
         <x:v>50</x:v>
       </x:c>
       <x:c r="B57" s="8" t="n">
-        <x:v>77</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C57" s="12" t="str">
-        <x:v>¿Contra qué selección marcó Messi su primer gol mundialista?</x:v>
+        <x:v>¿Quién era el entrenador argentino en el debut de Messi con la mayor?</x:v>
       </x:c>
       <x:c r="D57" s="12" t="str">
-        <x:v>México</x:v>
+        <x:v>José Pekerman</x:v>
       </x:c>
       <x:c r="E57" s="12" t="str">
-        <x:v>Costa de Marfil</x:v>
+        <x:v>Alfio Basile</x:v>
       </x:c>
       <x:c r="F57" s="12" t="str">
-        <x:v>Serbia y Montenegro</x:v>
+        <x:v>Diego Maradona</x:v>
       </x:c>
       <x:c r="G57" s="12" t="str">
-        <x:v>Países Bajos</x:v>
+        <x:v>Marcelo Bielsa</x:v>
       </x:c>
       <x:c r="H57" s="13" t="str">
-        <x:v>C</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I57" s="12" t="str">
-        <x:v>Marcó en el 6-0 de Argentina en 2006.</x:v>
+        <x:v>Pekerman lo convocó para su estreno en 2005.</x:v>
       </x:c>
       <x:c r="J57" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K57" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L57" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="62" customHeight="1">
+    <x:row r="58" ht="110" customHeight="1">
       <x:c r="A58" s="8" t="n">
         <x:v>51</x:v>
       </x:c>
       <x:c r="B58" s="8" t="n">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C58" s="12" t="str">
-        <x:v>¿Quién era el entrenador argentino en el debut de Messi con la mayor?</x:v>
+        <x:v>¿Contra qué selección hizo Messi su primer gol con la mayor?</x:v>
       </x:c>
       <x:c r="D58" s="12" t="str">
-        <x:v>José Pekerman</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E58" s="12" t="str">
-        <x:v>Alfio Basile</x:v>
+        <x:v>Croacia</x:v>
       </x:c>
       <x:c r="F58" s="12" t="str">
-        <x:v>Diego Maradona</x:v>
+        <x:v>Hungría</x:v>
       </x:c>
       <x:c r="G58" s="12" t="str">
-        <x:v>Marcelo Bielsa</x:v>
+        <x:v>Bolivia</x:v>
       </x:c>
       <x:c r="H58" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I58" s="12" t="str">
-        <x:v>Pekerman lo convocó para su estreno en 2005.</x:v>
+        <x:v>Anotó su primer gol ante Croacia en marzo de 2006.</x:v>
       </x:c>
       <x:c r="J58" s="12" t="str">
         <x:v>Intermedio</x:v>
@@ -2489,185 +2489,185 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" ht="62" customHeight="1">
+    <x:row r="59" ht="110" customHeight="1">
       <x:c r="A59" s="8" t="n">
         <x:v>52</x:v>
       </x:c>
       <x:c r="B59" s="8" t="n">
-        <x:v>54</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C59" s="12" t="str">
-        <x:v>¿Contra qué selección hizo Messi su primer gol con la mayor?</x:v>
+        <x:v>¿Cuántos goles hizo Messi en el Mundial 2010?</x:v>
       </x:c>
       <x:c r="D59" s="12" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E59" s="12" t="str">
-        <x:v>Croacia</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F59" s="12" t="str">
-        <x:v>Hungría</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G59" s="12" t="str">
-        <x:v>Bolivia</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H59" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I59" s="12" t="str">
-        <x:v>Anotó su primer gol ante Croacia en marzo de 2006.</x:v>
+        <x:v>No marcó en Sudáfrica, aunque sí participó en el ataque.</x:v>
       </x:c>
       <x:c r="J59" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K59" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L59" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" ht="62" customHeight="1">
+    <x:row r="60" ht="110" customHeight="1">
       <x:c r="A60" s="8" t="n">
         <x:v>53</x:v>
       </x:c>
       <x:c r="B60" s="8" t="n">
-        <x:v>80</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C60" s="12" t="str">
-        <x:v>¿Cuántos goles hizo Messi en el Mundial 2010?</x:v>
+        <x:v>¿A qué delantero superó Messi como goleador histórico de Argentina en 2016?</x:v>
       </x:c>
       <x:c r="D60" s="12" t="str">
-        <x:v>0</x:v>
+        <x:v>Mario Kempes</x:v>
       </x:c>
       <x:c r="E60" s="12" t="str">
-        <x:v>1</x:v>
+        <x:v>Gabriel Batistuta</x:v>
       </x:c>
       <x:c r="F60" s="12" t="str">
-        <x:v>4</x:v>
+        <x:v>Hernán Crespo</x:v>
       </x:c>
       <x:c r="G60" s="12" t="str">
-        <x:v>3</x:v>
+        <x:v>Claudio Caniggia</x:v>
       </x:c>
       <x:c r="H60" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I60" s="12" t="str">
-        <x:v>No marcó en Sudáfrica, aunque sí participó en el ataque.</x:v>
+        <x:v>Superó a Batistuta durante la Copa América Centenario.</x:v>
       </x:c>
       <x:c r="J60" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K60" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L60" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="62" customHeight="1">
+    <x:row r="61" ht="110" customHeight="1">
       <x:c r="A61" s="8" t="n">
         <x:v>54</x:v>
       </x:c>
       <x:c r="B61" s="8" t="n">
-        <x:v>56</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="C61" s="12" t="str">
-        <x:v>¿A qué delantero superó Messi como goleador histórico de Argentina en 2016?</x:v>
+        <x:v>¿Qué selección fue rival de Argentina en la final olímpica de 2008?</x:v>
       </x:c>
       <x:c r="D61" s="12" t="str">
-        <x:v>Mario Kempes</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E61" s="12" t="str">
-        <x:v>Gabriel Batistuta</x:v>
+        <x:v>Países Bajos</x:v>
       </x:c>
       <x:c r="F61" s="12" t="str">
-        <x:v>Hernán Crespo</x:v>
+        <x:v>Nigeria</x:v>
       </x:c>
       <x:c r="G61" s="12" t="str">
-        <x:v>Claudio Caniggia</x:v>
+        <x:v>Costa de Marfil</x:v>
       </x:c>
       <x:c r="H61" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I61" s="12" t="str">
-        <x:v>Superó a Batistuta durante la Copa América Centenario.</x:v>
+        <x:v>Argentina venció 1-0 a Nigeria.</x:v>
       </x:c>
       <x:c r="J61" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K61" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L61" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="62" ht="62" customHeight="1">
+    <x:row r="62" ht="110" customHeight="1">
       <x:c r="A62" s="8" t="n">
         <x:v>55</x:v>
       </x:c>
       <x:c r="B62" s="8" t="n">
-        <x:v>106</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C62" s="12" t="str">
-        <x:v>¿Qué selección fue rival de Argentina en la final olímpica de 2008?</x:v>
+        <x:v>¿Qué selección eliminó a la Argentina de Messi en cuartos de Sudáfrica 2010?</x:v>
       </x:c>
       <x:c r="D62" s="12" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="E62" s="12" t="str">
+        <x:v>Alemania</x:v>
+      </x:c>
+      <x:c r="F62" s="12" t="str">
+        <x:v>España</x:v>
+      </x:c>
+      <x:c r="G62" s="12" t="str">
         <x:v>Países Bajos</x:v>
       </x:c>
-      <x:c r="F62" s="12" t="str">
-        <x:v>Nigeria</x:v>
-      </x:c>
-      <x:c r="G62" s="12" t="str">
-        <x:v>Costa de Marfil</x:v>
-      </x:c>
       <x:c r="H62" s="13" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I62" s="12" t="str">
-        <x:v>Argentina venció 1-0 a Nigeria.</x:v>
+        <x:v>Alemania venció 4-0 a Argentina en los cuartos de final del Mundial de Sudáfrica 2010.</x:v>
       </x:c>
       <x:c r="J62" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K62" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L62" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63" ht="62" customHeight="1">
+        <x:v>https://www.afa.com.ar/primeraDivision/posts/historia-de-la-seleccion-argentina-en-los-mundiales</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="110" customHeight="1">
       <x:c r="A63" s="8" t="n">
         <x:v>56</x:v>
       </x:c>
       <x:c r="B63" s="8" t="n">
-        <x:v>32</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="C63" s="12" t="str">
-        <x:v>¿Qué selección eliminó a la Argentina de Messi en cuartos de Sudáfrica 2010?</x:v>
+        <x:v>¿Qué premio individual ganó Messi en el Mundial 2014?</x:v>
       </x:c>
       <x:c r="D63" s="12" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Bota de Oro</x:v>
       </x:c>
       <x:c r="E63" s="12" t="str">
-        <x:v>Alemania</x:v>
+        <x:v>Balón de Oro</x:v>
       </x:c>
       <x:c r="F63" s="12" t="str">
-        <x:v>España</x:v>
+        <x:v>Premio al mejor juvenil</x:v>
       </x:c>
       <x:c r="G63" s="12" t="str">
-        <x:v>Países Bajos</x:v>
+        <x:v>Guante de Oro</x:v>
       </x:c>
       <x:c r="H63" s="13" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="I63" s="12" t="str">
-        <x:v>Alemania venció 4-0 a Argentina en los cuartos de final del Mundial de Sudáfrica 2010.</x:v>
+        <x:v>Fue elegido mejor jugador de Brasil 2014.</x:v>
       </x:c>
       <x:c r="J63" s="12" t="str">
         <x:v>Intermedio</x:v>
@@ -2676,150 +2676,150 @@
         <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L63" s="11" t="str">
-        <x:v>https://www.afa.com.ar/primeraDivision/posts/historia-de-la-seleccion-argentina-en-los-mundiales</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64" ht="62" customHeight="1">
+        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="110" customHeight="1">
       <x:c r="A64" s="8" t="n">
         <x:v>57</x:v>
       </x:c>
       <x:c r="B64" s="8" t="n">
-        <x:v>82</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="C64" s="12" t="str">
-        <x:v>¿Qué premio individual ganó Messi en el Mundial 2014?</x:v>
+        <x:v>¿Quién hizo el gol de la final olímpica de 2008 tras un pase de Messi?</x:v>
       </x:c>
       <x:c r="D64" s="12" t="str">
-        <x:v>Bota de Oro</x:v>
+        <x:v>Ezequiel Lavezzi</x:v>
       </x:c>
       <x:c r="E64" s="12" t="str">
-        <x:v>Balón de Oro</x:v>
+        <x:v>Ángel Di María</x:v>
       </x:c>
       <x:c r="F64" s="12" t="str">
-        <x:v>Premio al mejor juvenil</x:v>
+        <x:v>Sergio Agüero</x:v>
       </x:c>
       <x:c r="G64" s="12" t="str">
-        <x:v>Guante de Oro</x:v>
+        <x:v>Juan Román Riquelme</x:v>
       </x:c>
       <x:c r="H64" s="13" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="I64" s="12" t="str">
-        <x:v>Fue elegido mejor jugador de Brasil 2014.</x:v>
+        <x:v>Di María definió por encima del arquero.</x:v>
       </x:c>
       <x:c r="J64" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K64" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L64" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="65" ht="62" customHeight="1">
+    <x:row r="65" ht="110" customHeight="1">
       <x:c r="A65" s="8" t="n">
         <x:v>58</x:v>
       </x:c>
       <x:c r="B65" s="8" t="n">
-        <x:v>107</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C65" s="12" t="str">
-        <x:v>¿Quién hizo el gol de la final olímpica de 2008 tras un pase de Messi?</x:v>
+        <x:v>¿Cómo terminó el partido del hat-trick de Messi en Quito en 2017?</x:v>
       </x:c>
       <x:c r="D65" s="12" t="str">
-        <x:v>Ezequiel Lavezzi</x:v>
+        <x:v>Empataron 3-3</x:v>
       </x:c>
       <x:c r="E65" s="12" t="str">
-        <x:v>Ángel Di María</x:v>
+        <x:v>Argentina ganó 3-0</x:v>
       </x:c>
       <x:c r="F65" s="12" t="str">
-        <x:v>Sergio Agüero</x:v>
+        <x:v>Argentina ganó 4-2</x:v>
       </x:c>
       <x:c r="G65" s="12" t="str">
-        <x:v>Juan Román Riquelme</x:v>
+        <x:v>Argentina ganó 3-1</x:v>
       </x:c>
       <x:c r="H65" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="I65" s="12" t="str">
-        <x:v>Di María definió por encima del arquero.</x:v>
+        <x:v>Argentina remontó el gol inicial de Ecuador y ganó 3-1.</x:v>
       </x:c>
       <x:c r="J65" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K65" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>El camino con Argentina</x:v>
       </x:c>
       <x:c r="L65" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="66" ht="62" customHeight="1">
+    <x:row r="66" ht="110" customHeight="1">
       <x:c r="A66" s="8" t="n">
         <x:v>59</x:v>
       </x:c>
       <x:c r="B66" s="8" t="n">
-        <x:v>9</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C66" s="12" t="str">
-        <x:v>¿Cómo terminó el partido del hat-trick de Messi en Quito en 2017?</x:v>
+        <x:v>¿Contra qué selección marcó Messi en el descuento para ganar 1-0 en 2014?</x:v>
       </x:c>
       <x:c r="D66" s="12" t="str">
-        <x:v>Empataron 3-3</x:v>
+        <x:v>Irán</x:v>
       </x:c>
       <x:c r="E66" s="12" t="str">
-        <x:v>Argentina ganó 3-0</x:v>
+        <x:v>Bélgica</x:v>
       </x:c>
       <x:c r="F66" s="12" t="str">
-        <x:v>Argentina ganó 4-2</x:v>
+        <x:v>Suiza</x:v>
       </x:c>
       <x:c r="G66" s="12" t="str">
-        <x:v>Argentina ganó 3-1</x:v>
+        <x:v>Argelia</x:v>
       </x:c>
       <x:c r="H66" s="13" t="str">
-        <x:v>D</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I66" s="12" t="str">
-        <x:v>Argentina remontó el gol inicial de Ecuador y ganó 3-1.</x:v>
+        <x:v>Su zurdazo decidió el partido contra Irán.</x:v>
       </x:c>
       <x:c r="J66" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K66" s="12" t="str">
-        <x:v>El camino con Argentina</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L66" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="67" ht="62" customHeight="1">
+    <x:row r="67" ht="110" customHeight="1">
       <x:c r="A67" s="8" t="n">
         <x:v>60</x:v>
       </x:c>
       <x:c r="B67" s="8" t="n">
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="C67" s="12" t="str">
-        <x:v>¿Contra qué selección marcó Messi en el descuento para ganar 1-0 en 2014?</x:v>
+        <x:v>¿Contra qué selección marcó Messi un doblete en la fase de grupos de Brasil 2014?</x:v>
       </x:c>
       <x:c r="D67" s="12" t="str">
-        <x:v>Irán</x:v>
+        <x:v>Ghana</x:v>
       </x:c>
       <x:c r="E67" s="12" t="str">
-        <x:v>Bélgica</x:v>
+        <x:v>Nigeria</x:v>
       </x:c>
       <x:c r="F67" s="12" t="str">
-        <x:v>Suiza</x:v>
+        <x:v>Camerún</x:v>
       </x:c>
       <x:c r="G67" s="12" t="str">
-        <x:v>Argelia</x:v>
+        <x:v>Costa de Marfil</x:v>
       </x:c>
       <x:c r="H67" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I67" s="12" t="str">
-        <x:v>Su zurdazo decidió el partido contra Irán.</x:v>
+        <x:v>Argentina venció 3-2 a Nigeria.</x:v>
       </x:c>
       <x:c r="J67" s="12" t="str">
         <x:v>Intermedio</x:v>
@@ -2831,527 +2831,527 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" ht="62" customHeight="1">
+    <x:row r="68" ht="110" customHeight="1">
       <x:c r="A68" s="8" t="n">
         <x:v>61</x:v>
       </x:c>
       <x:c r="B68" s="8" t="n">
-        <x:v>85</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C68" s="12" t="str">
-        <x:v>¿Contra qué selección marcó Messi un doblete en la fase de grupos de Brasil 2014?</x:v>
+        <x:v>¿En qué país se disputó la Copa América Centenario 2016 que jugó Messi?</x:v>
       </x:c>
       <x:c r="D68" s="12" t="str">
-        <x:v>Ghana</x:v>
+        <x:v>Estados Unidos</x:v>
       </x:c>
       <x:c r="E68" s="12" t="str">
-        <x:v>Nigeria</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="F68" s="12" t="str">
-        <x:v>Camerún</x:v>
+        <x:v>Chile</x:v>
       </x:c>
       <x:c r="G68" s="12" t="str">
-        <x:v>Costa de Marfil</x:v>
+        <x:v>Argentina</x:v>
       </x:c>
       <x:c r="H68" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I68" s="12" t="str">
-        <x:v>Argentina venció 3-2 a Nigeria.</x:v>
+        <x:v>La edición del centenario se jugó en Estados Unidos.</x:v>
       </x:c>
       <x:c r="J68" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K68" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L68" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="69" ht="62" customHeight="1">
+    <x:row r="69" ht="110" customHeight="1">
       <x:c r="A69" s="8" t="n">
         <x:v>62</x:v>
       </x:c>
       <x:c r="B69" s="8" t="n">
-        <x:v>110</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C69" s="12" t="str">
-        <x:v>¿En qué país se disputó la Copa América Centenario 2016 que jugó Messi?</x:v>
+        <x:v>¿Qué selección recibió el gol número 100 de Messi con Argentina en 2023?</x:v>
       </x:c>
       <x:c r="D69" s="12" t="str">
-        <x:v>Estados Unidos</x:v>
+        <x:v>Honduras</x:v>
       </x:c>
       <x:c r="E69" s="12" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Jamaica</x:v>
       </x:c>
       <x:c r="F69" s="12" t="str">
-        <x:v>Chile</x:v>
+        <x:v>Curazao</x:v>
       </x:c>
       <x:c r="G69" s="12" t="str">
-        <x:v>Argentina</x:v>
+        <x:v>Panamá</x:v>
       </x:c>
       <x:c r="H69" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I69" s="12" t="str">
-        <x:v>La edición del centenario se jugó en Estados Unidos.</x:v>
+        <x:v>Leo llegó al centenar de goles contra Curazao.</x:v>
       </x:c>
       <x:c r="J69" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K69" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L69" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" ht="62" customHeight="1">
+    <x:row r="70" ht="110" customHeight="1">
       <x:c r="A70" s="8" t="n">
         <x:v>63</x:v>
       </x:c>
       <x:c r="B70" s="8" t="n">
-        <x:v>61</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C70" s="12" t="str">
-        <x:v>¿Qué selección recibió el gol número 100 de Messi con Argentina en 2023?</x:v>
+        <x:v>¿En qué edición jugó Messi su primera Copa América?</x:v>
       </x:c>
       <x:c r="D70" s="12" t="str">
-        <x:v>Honduras</x:v>
+        <x:v>Venezuela 2007</x:v>
       </x:c>
       <x:c r="E70" s="12" t="str">
-        <x:v>Jamaica</x:v>
+        <x:v>Argentina 2011</x:v>
       </x:c>
       <x:c r="F70" s="12" t="str">
-        <x:v>Curazao</x:v>
+        <x:v>Chile 2015</x:v>
       </x:c>
       <x:c r="G70" s="12" t="str">
-        <x:v>Panamá</x:v>
+        <x:v>Perú 2004</x:v>
       </x:c>
       <x:c r="H70" s="13" t="str">
-        <x:v>C</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I70" s="12" t="str">
-        <x:v>Leo llegó al centenar de goles contra Curazao.</x:v>
+        <x:v>Su primera participación fue en Venezuela 2007.</x:v>
       </x:c>
       <x:c r="J70" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K70" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>El camino con Argentina</x:v>
       </x:c>
       <x:c r="L70" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" ht="62" customHeight="1">
+    <x:row r="71" ht="110" customHeight="1">
       <x:c r="A71" s="8" t="n">
         <x:v>64</x:v>
       </x:c>
       <x:c r="B71" s="8" t="n">
-        <x:v>12</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="C71" s="12" t="str">
-        <x:v>¿En qué edición jugó Messi su primera Copa América?</x:v>
+        <x:v>¿En qué grupo jugó Argentina con Messi en Qatar 2022?</x:v>
       </x:c>
       <x:c r="D71" s="12" t="str">
-        <x:v>Venezuela 2007</x:v>
+        <x:v>Grupo C</x:v>
       </x:c>
       <x:c r="E71" s="12" t="str">
-        <x:v>Argentina 2011</x:v>
+        <x:v>Grupo D</x:v>
       </x:c>
       <x:c r="F71" s="12" t="str">
-        <x:v>Chile 2015</x:v>
+        <x:v>Grupo A</x:v>
       </x:c>
       <x:c r="G71" s="12" t="str">
-        <x:v>Perú 2004</x:v>
+        <x:v>Grupo B</x:v>
       </x:c>
       <x:c r="H71" s="13" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="I71" s="12" t="str">
-        <x:v>Su primera participación fue en Venezuela 2007.</x:v>
+        <x:v>Compartió el grupo C con Arabia Saudita, México y Polonia.</x:v>
       </x:c>
       <x:c r="J71" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K71" s="12" t="str">
-        <x:v>El camino con Argentina</x:v>
+        <x:v>Qatar en detalle</x:v>
       </x:c>
       <x:c r="L71" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="72" ht="62" customHeight="1">
+    <x:row r="72" ht="110" customHeight="1">
       <x:c r="A72" s="8" t="n">
         <x:v>65</x:v>
       </x:c>
       <x:c r="B72" s="8" t="n">
-        <x:v>37</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="C72" s="12" t="str">
-        <x:v>¿En qué grupo jugó Argentina con Messi en Qatar 2022?</x:v>
+        <x:v>¿Contra qué selección marcó Messi su único gol en Rusia 2018?</x:v>
       </x:c>
       <x:c r="D72" s="12" t="str">
-        <x:v>Grupo C</x:v>
+        <x:v>Islandia</x:v>
       </x:c>
       <x:c r="E72" s="12" t="str">
-        <x:v>Grupo D</x:v>
+        <x:v>Croacia</x:v>
       </x:c>
       <x:c r="F72" s="12" t="str">
-        <x:v>Grupo A</x:v>
+        <x:v>Nigeria</x:v>
       </x:c>
       <x:c r="G72" s="12" t="str">
-        <x:v>Grupo B</x:v>
+        <x:v>Francia</x:v>
       </x:c>
       <x:c r="H72" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I72" s="12" t="str">
-        <x:v>Compartió el grupo C con Arabia Saudita, México y Polonia.</x:v>
+        <x:v>Abrió el marcador en el triunfo 2-1 sobre Nigeria.</x:v>
       </x:c>
       <x:c r="J72" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K72" s="12" t="str">
-        <x:v>Qatar en detalle</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L72" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="73" ht="62" customHeight="1">
+    <x:row r="73" ht="110" customHeight="1">
       <x:c r="A73" s="8" t="n">
         <x:v>66</x:v>
       </x:c>
       <x:c r="B73" s="8" t="n">
-        <x:v>87</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C73" s="12" t="str">
-        <x:v>¿Contra qué selección marcó Messi su único gol en Rusia 2018?</x:v>
+        <x:v>¿Contra qué selección marcó Messi de globito en la semifinal de la Copa América 2007?</x:v>
       </x:c>
       <x:c r="D73" s="12" t="str">
-        <x:v>Islandia</x:v>
+        <x:v>Uruguay</x:v>
       </x:c>
       <x:c r="E73" s="12" t="str">
-        <x:v>Croacia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="F73" s="12" t="str">
-        <x:v>Nigeria</x:v>
+        <x:v>México</x:v>
       </x:c>
       <x:c r="G73" s="12" t="str">
-        <x:v>Francia</x:v>
+        <x:v>Paraguay</x:v>
       </x:c>
       <x:c r="H73" s="13" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="I73" s="12" t="str">
-        <x:v>Abrió el marcador en el triunfo 2-1 sobre Nigeria.</x:v>
+        <x:v>Leo elevó la pelota sobre Oswaldo Sánchez en el 3-0 a México.</x:v>
       </x:c>
       <x:c r="J73" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K73" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>El camino con Argentina</x:v>
       </x:c>
       <x:c r="L73" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="74" ht="62" customHeight="1">
+    <x:row r="74" ht="110" customHeight="1">
       <x:c r="A74" s="8" t="n">
         <x:v>67</x:v>
       </x:c>
       <x:c r="B74" s="8" t="n">
-        <x:v>13</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C74" s="12" t="str">
-        <x:v>¿Contra qué selección marcó Messi de globito en la semifinal de la Copa América 2007?</x:v>
+        <x:v>¿Qué selección recibió un hat-trick de Messi en un 4-3 de 2012?</x:v>
       </x:c>
       <x:c r="D74" s="12" t="str">
-        <x:v>Uruguay</x:v>
+        <x:v>España</x:v>
       </x:c>
       <x:c r="E74" s="12" t="str">
         <x:v>Brasil</x:v>
       </x:c>
       <x:c r="F74" s="12" t="str">
-        <x:v>México</x:v>
+        <x:v>Alemania</x:v>
       </x:c>
       <x:c r="G74" s="12" t="str">
-        <x:v>Paraguay</x:v>
+        <x:v>Italia</x:v>
       </x:c>
       <x:c r="H74" s="13" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I74" s="12" t="str">
-        <x:v>Leo elevó la pelota sobre Oswaldo Sánchez en el 3-0 a México.</x:v>
+        <x:v>Messi marcó tres veces en el amistoso ante Brasil.</x:v>
       </x:c>
       <x:c r="J74" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K74" s="12" t="str">
-        <x:v>El camino con Argentina</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L74" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="75" ht="62" customHeight="1">
+    <x:row r="75" ht="110" customHeight="1">
       <x:c r="A75" s="8" t="n">
         <x:v>68</x:v>
       </x:c>
       <x:c r="B75" s="8" t="n">
-        <x:v>63</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C75" s="12" t="str">
-        <x:v>¿Qué selección recibió un hat-trick de Messi en un 4-3 de 2012?</x:v>
+        <x:v>¿Contra qué selección fue eliminada la Argentina de Messi en la Copa América 2011?</x:v>
       </x:c>
       <x:c r="D75" s="12" t="str">
-        <x:v>España</x:v>
+        <x:v>Uruguay</x:v>
       </x:c>
       <x:c r="E75" s="12" t="str">
+        <x:v>Colombia</x:v>
+      </x:c>
+      <x:c r="F75" s="12" t="str">
+        <x:v>Chile</x:v>
+      </x:c>
+      <x:c r="G75" s="12" t="str">
         <x:v>Brasil</x:v>
       </x:c>
-      <x:c r="F75" s="12" t="str">
-        <x:v>Alemania</x:v>
-      </x:c>
-      <x:c r="G75" s="12" t="str">
-        <x:v>Italia</x:v>
-      </x:c>
       <x:c r="H75" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I75" s="12" t="str">
-        <x:v>Messi marcó tres veces en el amistoso ante Brasil.</x:v>
+        <x:v>Uruguay se impuso por penales en cuartos de final.</x:v>
       </x:c>
       <x:c r="J75" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K75" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>El camino con Argentina</x:v>
       </x:c>
       <x:c r="L75" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="76" ht="62" customHeight="1">
+    <x:row r="76" ht="110" customHeight="1">
       <x:c r="A76" s="8" t="n">
         <x:v>69</x:v>
       </x:c>
       <x:c r="B76" s="8" t="n">
-        <x:v>14</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C76" s="12" t="str">
-        <x:v>¿Contra qué selección fue eliminada la Argentina de Messi en la Copa América 2011?</x:v>
+        <x:v>¿Contra qué selección hizo Messi un hat-trick en el Monumental en septiembre de 2021?</x:v>
       </x:c>
       <x:c r="D76" s="12" t="str">
-        <x:v>Uruguay</x:v>
+        <x:v>Perú</x:v>
       </x:c>
       <x:c r="E76" s="12" t="str">
-        <x:v>Colombia</x:v>
+        <x:v>Venezuela</x:v>
       </x:c>
       <x:c r="F76" s="12" t="str">
-        <x:v>Chile</x:v>
+        <x:v>Bolivia</x:v>
       </x:c>
       <x:c r="G76" s="12" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>Paraguay</x:v>
       </x:c>
       <x:c r="H76" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I76" s="12" t="str">
-        <x:v>Uruguay se impuso por penales en cuartos de final.</x:v>
+        <x:v>El encuentro terminó 3-0 para Argentina.</x:v>
       </x:c>
       <x:c r="J76" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K76" s="12" t="str">
-        <x:v>El camino con Argentina</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L76" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="77" ht="62" customHeight="1">
+    <x:row r="77" ht="110" customHeight="1">
       <x:c r="A77" s="8" t="n">
         <x:v>70</x:v>
       </x:c>
       <x:c r="B77" s="8" t="n">
-        <x:v>64</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C77" s="12" t="str">
-        <x:v>¿Contra qué selección hizo Messi un hat-trick en el Monumental en septiembre de 2021?</x:v>
+        <x:v>¿A qué selección le ganó Argentina 6-1 en la semifinal de la Copa América 2015, con Messi como figura?</x:v>
       </x:c>
       <x:c r="D77" s="12" t="str">
+        <x:v>Bolivia</x:v>
+      </x:c>
+      <x:c r="E77" s="12" t="str">
         <x:v>Perú</x:v>
       </x:c>
-      <x:c r="E77" s="12" t="str">
-        <x:v>Venezuela</x:v>
-      </x:c>
       <x:c r="F77" s="12" t="str">
-        <x:v>Bolivia</x:v>
+        <x:v>Paraguay</x:v>
       </x:c>
       <x:c r="G77" s="12" t="str">
-        <x:v>Paraguay</x:v>
+        <x:v>Ecuador</x:v>
       </x:c>
       <x:c r="H77" s="13" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="I77" s="12" t="str">
-        <x:v>El encuentro terminó 3-0 para Argentina.</x:v>
+        <x:v>El equipo argentino goleó a Paraguay para llegar a la final.</x:v>
       </x:c>
       <x:c r="J77" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K77" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>El camino con Argentina</x:v>
       </x:c>
       <x:c r="L77" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="78" ht="62" customHeight="1">
+    <x:row r="78" ht="110" customHeight="1">
       <x:c r="A78" s="8" t="n">
         <x:v>71</x:v>
       </x:c>
       <x:c r="B78" s="8" t="n">
-        <x:v>15</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C78" s="12" t="str">
-        <x:v>¿A qué selección le ganó Argentina 6-1 en la semifinal de la Copa América 2015, con Messi como figura?</x:v>
+        <x:v>¿Qué técnico nombró a Messi capitán de Argentina en 2011?</x:v>
       </x:c>
       <x:c r="D78" s="12" t="str">
-        <x:v>Bolivia</x:v>
+        <x:v>Jorge Sampaoli</x:v>
       </x:c>
       <x:c r="E78" s="12" t="str">
-        <x:v>Perú</x:v>
+        <x:v>José Pekerman</x:v>
       </x:c>
       <x:c r="F78" s="12" t="str">
-        <x:v>Paraguay</x:v>
+        <x:v>Alejandro Sabella</x:v>
       </x:c>
       <x:c r="G78" s="12" t="str">
-        <x:v>Ecuador</x:v>
+        <x:v>Diego Maradona</x:v>
       </x:c>
       <x:c r="H78" s="13" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="I78" s="12" t="str">
-        <x:v>El equipo argentino goleó a Paraguay para llegar a la final.</x:v>
+        <x:v>Sabella le dio la capitanía al asumir.</x:v>
       </x:c>
       <x:c r="J78" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K78" s="12" t="str">
-        <x:v>El camino con Argentina</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L78" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="79" ht="62" customHeight="1">
+    <x:row r="79" ht="110" customHeight="1">
       <x:c r="A79" s="8" t="n">
         <x:v>72</x:v>
       </x:c>
       <x:c r="B79" s="8" t="n">
-        <x:v>66</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="C79" s="12" t="str">
-        <x:v>¿Qué técnico nombró a Messi capitán de Argentina en 2011?</x:v>
+        <x:v>¿Cuántos goles hizo Messi en la Copa América 2021?</x:v>
       </x:c>
       <x:c r="D79" s="12" t="str">
-        <x:v>Jorge Sampaoli</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E79" s="12" t="str">
-        <x:v>José Pekerman</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F79" s="12" t="str">
-        <x:v>Alejandro Sabella</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G79" s="12" t="str">
-        <x:v>Diego Maradona</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H79" s="13" t="str">
-        <x:v>C</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I79" s="12" t="str">
-        <x:v>Sabella le dio la capitanía al asumir.</x:v>
+        <x:v>Messi terminó el torneo con cuatro goles.</x:v>
       </x:c>
       <x:c r="J79" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K79" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L79" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="80" ht="62" customHeight="1">
+    <x:row r="80" ht="110" customHeight="1">
       <x:c r="A80" s="8" t="n">
         <x:v>73</x:v>
       </x:c>
       <x:c r="B80" s="8" t="n">
-        <x:v>117</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C80" s="12" t="str">
-        <x:v>¿Cuántos goles hizo Messi en la Copa América 2021?</x:v>
+        <x:v>¿Contra qué selección jugó Argentina su primer partido de Brasil 2014?</x:v>
       </x:c>
       <x:c r="D80" s="12" t="str">
-        <x:v>4</x:v>
+        <x:v>Nigeria</x:v>
       </x:c>
       <x:c r="E80" s="12" t="str">
-        <x:v>6</x:v>
+        <x:v>Irán</x:v>
       </x:c>
       <x:c r="F80" s="12" t="str">
-        <x:v>2</x:v>
+        <x:v>Croacia</x:v>
       </x:c>
       <x:c r="G80" s="12" t="str">
-        <x:v>5</x:v>
+        <x:v>Bosnia y Herzegovina</x:v>
       </x:c>
       <x:c r="H80" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="I80" s="12" t="str">
-        <x:v>Messi terminó el torneo con cuatro goles.</x:v>
+        <x:v>Argentina debutó con un triunfo 2-1 ante Bosnia y Herzegovina. Messi marcó el segundo gol argentino.</x:v>
       </x:c>
       <x:c r="J80" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K80" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L80" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="81" ht="62" customHeight="1">
+        <x:v>https://www.fifa.com/es/tournaments/mens/worldcup</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="110" customHeight="1">
       <x:c r="A81" s="8" t="n">
         <x:v>74</x:v>
       </x:c>
       <x:c r="B81" s="8" t="n">
-        <x:v>18</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="C81" s="12" t="str">
-        <x:v>¿Contra qué selección jugó Argentina su primer partido de Brasil 2014?</x:v>
+        <x:v>¿A qué jugador asistió Messi en el primer gol contra Países Bajos en Qatar?</x:v>
       </x:c>
       <x:c r="D81" s="12" t="str">
-        <x:v>Nigeria</x:v>
+        <x:v>Marcos Acuña</x:v>
       </x:c>
       <x:c r="E81" s="12" t="str">
-        <x:v>Irán</x:v>
+        <x:v>Cristian Romero</x:v>
       </x:c>
       <x:c r="F81" s="12" t="str">
-        <x:v>Croacia</x:v>
+        <x:v>Nicolás Otamendi</x:v>
       </x:c>
       <x:c r="G81" s="12" t="str">
-        <x:v>Bosnia y Herzegovina</x:v>
+        <x:v>Nahuel Molina</x:v>
       </x:c>
       <x:c r="H81" s="13" t="str">
         <x:v>D</x:v>
       </x:c>
       <x:c r="I81" s="12" t="str">
-        <x:v>Argentina debutó con un triunfo 2-1 ante Bosnia y Herzegovina. Messi marcó el segundo gol argentino.</x:v>
+        <x:v>Molina marcó tras un pase de Leo entre defensores.</x:v>
       </x:c>
       <x:c r="J81" s="12" t="str">
         <x:v>Intermedio</x:v>
@@ -3360,112 +3360,112 @@
         <x:v>Los Mundiales</x:v>
       </x:c>
       <x:c r="L81" s="11" t="str">
-        <x:v>https://www.fifa.com/es/tournaments/mens/worldcup</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="82" ht="62" customHeight="1">
+        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="110" customHeight="1">
       <x:c r="A82" s="8" t="n">
         <x:v>75</x:v>
       </x:c>
       <x:c r="B82" s="8" t="n">
-        <x:v>93</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C82" s="12" t="str">
-        <x:v>¿A qué jugador asistió Messi en el primer gol contra Países Bajos en Qatar?</x:v>
+        <x:v>¿Qué selección recibió un gol de Messi en el amistoso que Argentina ganó 4-1 en 2010?</x:v>
       </x:c>
       <x:c r="D82" s="12" t="str">
-        <x:v>Marcos Acuña</x:v>
+        <x:v>España</x:v>
       </x:c>
       <x:c r="E82" s="12" t="str">
-        <x:v>Cristian Romero</x:v>
+        <x:v>Francia</x:v>
       </x:c>
       <x:c r="F82" s="12" t="str">
-        <x:v>Nicolás Otamendi</x:v>
+        <x:v>Portugal</x:v>
       </x:c>
       <x:c r="G82" s="12" t="str">
-        <x:v>Nahuel Molina</x:v>
+        <x:v>Italia</x:v>
       </x:c>
       <x:c r="H82" s="13" t="str">
-        <x:v>D</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I82" s="12" t="str">
-        <x:v>Molina marcó tras un pase de Leo entre defensores.</x:v>
+        <x:v>Messi abrió el marcador ante la campeona mundial España.</x:v>
       </x:c>
       <x:c r="J82" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K82" s="12" t="str">
-        <x:v>Los Mundiales</x:v>
+        <x:v>El camino con Argentina</x:v>
       </x:c>
       <x:c r="L82" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="83" ht="62" customHeight="1">
+    <x:row r="83" ht="110" customHeight="1">
       <x:c r="A83" s="8" t="n">
         <x:v>76</x:v>
       </x:c>
       <x:c r="B83" s="8" t="n">
-        <x:v>19</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C83" s="12" t="str">
-        <x:v>¿Qué selección recibió un gol de Messi en el amistoso que Argentina ganó 4-1 en 2010?</x:v>
+        <x:v>¿Qué selección recibió un hat-trick de Messi en el 6-0 de octubre de 2024?</x:v>
       </x:c>
       <x:c r="D83" s="12" t="str">
-        <x:v>España</x:v>
+        <x:v>Colombia</x:v>
       </x:c>
       <x:c r="E83" s="12" t="str">
-        <x:v>Francia</x:v>
+        <x:v>Uruguay</x:v>
       </x:c>
       <x:c r="F83" s="12" t="str">
-        <x:v>Portugal</x:v>
+        <x:v>Paraguay</x:v>
       </x:c>
       <x:c r="G83" s="12" t="str">
-        <x:v>Italia</x:v>
+        <x:v>Bolivia</x:v>
       </x:c>
       <x:c r="H83" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="I83" s="12" t="str">
-        <x:v>Messi abrió el marcador ante la campeona mundial España.</x:v>
+        <x:v>Leo marcó tres veces en el Monumental ante Bolivia.</x:v>
       </x:c>
       <x:c r="J83" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K83" s="12" t="str">
-        <x:v>El camino con Argentina</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L83" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="84" ht="62" customHeight="1">
+    <x:row r="84" ht="110" customHeight="1">
       <x:c r="A84" s="8" t="n">
         <x:v>77</x:v>
       </x:c>
       <x:c r="B84" s="8" t="n">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C84" s="12" t="str">
-        <x:v>¿Qué selección recibió un hat-trick de Messi en el 6-0 de octubre de 2024?</x:v>
+        <x:v>¿Qué selección recibió un tiro libre de Messi en el 1-0 de septiembre de 2023 en el inicio de las eliminatorias?</x:v>
       </x:c>
       <x:c r="D84" s="12" t="str">
-        <x:v>Colombia</x:v>
+        <x:v>Uruguay</x:v>
       </x:c>
       <x:c r="E84" s="12" t="str">
-        <x:v>Uruguay</x:v>
+        <x:v>Chile</x:v>
       </x:c>
       <x:c r="F84" s="12" t="str">
-        <x:v>Paraguay</x:v>
+        <x:v>Ecuador</x:v>
       </x:c>
       <x:c r="G84" s="12" t="str">
-        <x:v>Bolivia</x:v>
+        <x:v>Brasil</x:v>
       </x:c>
       <x:c r="H84" s="13" t="str">
-        <x:v>D</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I84" s="12" t="str">
-        <x:v>Leo marcó tres veces en el Monumental ante Bolivia.</x:v>
+        <x:v>Messi decidió el inicio de las Eliminatorias con un tiro libre.</x:v>
       </x:c>
       <x:c r="J84" s="12" t="str">
         <x:v>Intermedio</x:v>
@@ -3477,223 +3477,223 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="85" ht="62" customHeight="1">
+    <x:row r="85" ht="110" customHeight="1">
       <x:c r="A85" s="8" t="n">
         <x:v>78</x:v>
       </x:c>
       <x:c r="B85" s="8" t="n">
-        <x:v>71</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C85" s="12" t="str">
-        <x:v>¿Qué selección recibió un tiro libre de Messi en el 1-0 de septiembre de 2023 en el inicio de las eliminatorias?</x:v>
+        <x:v>¿Hacia qué lado remató Messi, desde su perspectiva, en la tanda de la final de Qatar 2022?</x:v>
       </x:c>
       <x:c r="D85" s="12" t="str">
-        <x:v>Uruguay</x:v>
+        <x:v>Al centro del arco</x:v>
       </x:c>
       <x:c r="E85" s="12" t="str">
-        <x:v>Chile</x:v>
+        <x:v>La picó por encima del arquero</x:v>
       </x:c>
       <x:c r="F85" s="12" t="str">
-        <x:v>Ecuador</x:v>
+        <x:v>A su izquierda</x:v>
       </x:c>
       <x:c r="G85" s="12" t="str">
-        <x:v>Brasil</x:v>
+        <x:v>A su derecha</x:v>
       </x:c>
       <x:c r="H85" s="13" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="I85" s="12" t="str">
-        <x:v>Messi decidió el inicio de las Eliminatorias con un tiro libre.</x:v>
+        <x:v>Messi remató bajo a su izquierda, desde la perspectiva del ejecutante, y convirtió el primer penal argentino de la tanda.</x:v>
       </x:c>
       <x:c r="J85" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K85" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>Qatar en detalle</x:v>
       </x:c>
       <x:c r="L85" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="86" ht="62" customHeight="1">
+        <x:v>https://www.laliga.com/partido/temporada-2022-2023-mundial-fifa-qatar-2022-argentina-francia-8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="110" customHeight="1">
       <x:c r="A86" s="8" t="n">
         <x:v>79</x:v>
       </x:c>
       <x:c r="B86" s="8" t="n">
-        <x:v>47</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C86" s="12" t="str">
-        <x:v>¿Hacia qué lado remató Messi, desde su perspectiva, en la tanda de la final de Qatar 2022?</x:v>
+        <x:v>¿Contra qué selección marcó Messi de tiro libre en el amistoso de marzo de 2023?</x:v>
       </x:c>
       <x:c r="D86" s="12" t="str">
-        <x:v>Al centro del arco</x:v>
+        <x:v>China</x:v>
       </x:c>
       <x:c r="E86" s="12" t="str">
-        <x:v>La picó por encima del arquero</x:v>
+        <x:v>Panamá</x:v>
       </x:c>
       <x:c r="F86" s="12" t="str">
-        <x:v>A su izquierda</x:v>
+        <x:v>México</x:v>
       </x:c>
       <x:c r="G86" s="12" t="str">
-        <x:v>A su derecha</x:v>
+        <x:v>Estados Unidos</x:v>
       </x:c>
       <x:c r="H86" s="13" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="I86" s="12" t="str">
-        <x:v>Messi remató bajo a su izquierda, desde la perspectiva del ejecutante, y convirtió el primer penal argentino de la tanda.</x:v>
+        <x:v>El partido ante Panamá terminó 2-0 para Argentina.</x:v>
       </x:c>
       <x:c r="J86" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K86" s="12" t="str">
-        <x:v>Qatar en detalle</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L86" s="11" t="str">
-        <x:v>https://www.laliga.com/partido/temporada-2022-2023-mundial-fifa-qatar-2022-argentina-francia-8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="87" ht="62" customHeight="1">
+        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="110" customHeight="1">
       <x:c r="A87" s="8" t="n">
         <x:v>80</x:v>
       </x:c>
       <x:c r="B87" s="8" t="n">
-        <x:v>72</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C87" s="12" t="str">
-        <x:v>¿Contra qué selección marcó Messi de tiro libre en el amistoso de marzo de 2023?</x:v>
+        <x:v>¿Contra qué selección convirtió Messi de tiro libre en cuartos de la Copa América 2021?</x:v>
       </x:c>
       <x:c r="D87" s="12" t="str">
-        <x:v>China</x:v>
+        <x:v>Ecuador</x:v>
       </x:c>
       <x:c r="E87" s="12" t="str">
-        <x:v>Panamá</x:v>
+        <x:v>Venezuela</x:v>
       </x:c>
       <x:c r="F87" s="12" t="str">
-        <x:v>México</x:v>
+        <x:v>Uruguay</x:v>
       </x:c>
       <x:c r="G87" s="12" t="str">
-        <x:v>Estados Unidos</x:v>
+        <x:v>Colombia</x:v>
       </x:c>
       <x:c r="H87" s="13" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I87" s="12" t="str">
-        <x:v>El partido ante Panamá terminó 2-0 para Argentina.</x:v>
+        <x:v>Su tiro libre cerró el 3-0 ante Ecuador.</x:v>
       </x:c>
       <x:c r="J87" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K87" s="12" t="str">
-        <x:v>La Albiceleste</x:v>
+        <x:v>El camino con Argentina</x:v>
       </x:c>
       <x:c r="L87" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="88" ht="62" customHeight="1">
+    <x:row r="88" ht="110" customHeight="1">
       <x:c r="A88" s="8" t="n">
         <x:v>81</x:v>
       </x:c>
       <x:c r="B88" s="8" t="n">
-        <x:v>23</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="C88" s="12" t="str">
-        <x:v>¿Contra qué selección convirtió Messi de tiro libre en cuartos de la Copa América 2021?</x:v>
+        <x:v>¿Contra qué selección marcó Messi en la semifinal de la Copa América 2024?</x:v>
       </x:c>
       <x:c r="D88" s="12" t="str">
-        <x:v>Ecuador</x:v>
+        <x:v>México</x:v>
       </x:c>
       <x:c r="E88" s="12" t="str">
-        <x:v>Venezuela</x:v>
+        <x:v>Chile</x:v>
       </x:c>
       <x:c r="F88" s="12" t="str">
-        <x:v>Uruguay</x:v>
+        <x:v>Estados Unidos</x:v>
       </x:c>
       <x:c r="G88" s="12" t="str">
-        <x:v>Colombia</x:v>
+        <x:v>Canadá</x:v>
       </x:c>
       <x:c r="H88" s="13" t="str">
-        <x:v>A</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="I88" s="12" t="str">
-        <x:v>Su tiro libre cerró el 3-0 ante Ecuador.</x:v>
+        <x:v>Messi anotó en el 2-0 sobre Canadá.</x:v>
       </x:c>
       <x:c r="J88" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K88" s="12" t="str">
-        <x:v>El camino con Argentina</x:v>
+        <x:v>Títulos y momentos</x:v>
       </x:c>
       <x:c r="L88" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="89" ht="62" customHeight="1">
+    <x:row r="89" ht="110" customHeight="1">
       <x:c r="A89" s="8" t="n">
         <x:v>82</x:v>
       </x:c>
       <x:c r="B89" s="8" t="n">
-        <x:v>123</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C89" s="12" t="str">
-        <x:v>¿Contra qué selección marcó Messi en la semifinal de la Copa América 2024?</x:v>
+        <x:v>¿Contra qué selección anotó Messi de tiro libre en el debut de la Copa América 2021?</x:v>
       </x:c>
       <x:c r="D89" s="12" t="str">
-        <x:v>México</x:v>
+        <x:v>Paraguay</x:v>
       </x:c>
       <x:c r="E89" s="12" t="str">
+        <x:v>Uruguay</x:v>
+      </x:c>
+      <x:c r="F89" s="12" t="str">
         <x:v>Chile</x:v>
       </x:c>
-      <x:c r="F89" s="12" t="str">
-        <x:v>Estados Unidos</x:v>
-      </x:c>
       <x:c r="G89" s="12" t="str">
-        <x:v>Canadá</x:v>
+        <x:v>Bolivia</x:v>
       </x:c>
       <x:c r="H89" s="13" t="str">
-        <x:v>D</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I89" s="12" t="str">
-        <x:v>Messi anotó en el 2-0 sobre Canadá.</x:v>
+        <x:v>El partido terminó 1-1 frente a Chile.</x:v>
       </x:c>
       <x:c r="J89" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K89" s="12" t="str">
-        <x:v>Títulos y momentos</x:v>
+        <x:v>El camino con Argentina</x:v>
       </x:c>
       <x:c r="L89" s="11" t="str">
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="90" ht="62" customHeight="1">
+    <x:row r="90" ht="110" customHeight="1">
       <x:c r="A90" s="8" t="n">
         <x:v>83</x:v>
       </x:c>
       <x:c r="B90" s="8" t="n">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C90" s="12" t="str">
-        <x:v>¿Contra qué selección anotó Messi de tiro libre en el debut de la Copa América 2021?</x:v>
+        <x:v>¿Contra qué selección hizo Messi dos goles en el último partido del grupo de la Copa América 2021?</x:v>
       </x:c>
       <x:c r="D90" s="12" t="str">
         <x:v>Paraguay</x:v>
       </x:c>
       <x:c r="E90" s="12" t="str">
+        <x:v>Chile</x:v>
+      </x:c>
+      <x:c r="F90" s="12" t="str">
         <x:v>Uruguay</x:v>
-      </x:c>
-      <x:c r="F90" s="12" t="str">
-        <x:v>Chile</x:v>
       </x:c>
       <x:c r="G90" s="12" t="str">
         <x:v>Bolivia</x:v>
       </x:c>
       <x:c r="H90" s="13" t="str">
-        <x:v>C</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="I90" s="12" t="str">
-        <x:v>El partido terminó 1-1 frente a Chile.</x:v>
+        <x:v>Argentina ganó 4-1 a Bolivia con un doblete del capitán.</x:v>
       </x:c>
       <x:c r="J90" s="12" t="str">
         <x:v>Intermedio</x:v>
@@ -3705,80 +3705,80 @@
         <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" ht="62" customHeight="1">
+    <x:row r="91" ht="110" customHeight="1">
       <x:c r="A91" s="8" t="n">
         <x:v>84</x:v>
       </x:c>
       <x:c r="B91" s="8" t="n">
-        <x:v>25</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C91" s="12" t="str">
-        <x:v>¿Contra qué selección hizo Messi dos goles en el último partido del grupo de la Copa América 2021?</x:v>
+        <x:v>¿Cuántos goles de tiro libre con la Selección registra Messi en la edición de octubre de 2026?</x:v>
       </x:c>
       <x:c r="D91" s="12" t="str">
-        <x:v>Paraguay</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E91" s="12" t="str">
-        <x:v>Chile</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F91" s="12" t="str">
-        <x:v>Uruguay</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G91" s="12" t="str">
-        <x:v>Bolivia</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H91" s="13" t="str">
-        <x:v>D</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I91" s="12" t="str">
-        <x:v>Argentina ganó 4-1 a Bolivia con un doblete del capitán.</x:v>
+        <x:v>La referencia usada para esta edición registra 12 goles de tiro libre de Messi con la Selección Argentina.</x:v>
       </x:c>
       <x:c r="J91" s="12" t="str">
         <x:v>Intermedio</x:v>
       </x:c>
       <x:c r="K91" s="12" t="str">
-        <x:v>El camino con Argentina</x:v>
+        <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L91" s="11" t="str">
-        <x:v>https://github.com/GB-Films/QUIZ-MESSI/blob/main/dist/questions.js</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="92" ht="62" customHeight="1">
+        <x:v>https://es.mlssoccer.com/noticias/messi-maradona-y-una-postal-bles-inolvidables-en-sunday-night-soccer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="110" customHeight="1">
       <x:c r="A92" s="8" t="n">
         <x:v>85</x:v>
       </x:c>
       <x:c r="B92" s="8" t="n">
-        <x:v>75</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="C92" s="12" t="str">
-        <x:v>¿Cuántos goles de tiro libre con la Selección registra Messi en la edición de octubre de 2026?</x:v>
+        <x:v>Según el balance de la AFA de octubre de 2026, ¿cuántas asistencias acumuló Messi con la Selección mayor?</x:v>
       </x:c>
       <x:c r="D92" s="12" t="str">
-        <x:v>8</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E92" s="12" t="str">
-        <x:v>10</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F92" s="12" t="str">
-        <x:v>12</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="G92" s="12" t="str">
-        <x:v>16</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="H92" s="13" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="I92" s="12" t="str">
-        <x:v>La referencia usada para esta edición registra 12 goles de tiro libre de Messi con la Selección Argentina.</x:v>
+        <x:v>El balance publicado por la AFA el 5 de octubre de 2026 registra 66 asistencias en 207 partidos con la Selección mayor. Esta pregunta usa esa fuente y esa fecha, porque otras estadísticas pueden contar las asistencias de manera diferente.</x:v>
       </x:c>
       <x:c r="J92" s="12" t="str">
-        <x:v>Intermedio</x:v>
+        <x:v>Difícil</x:v>
       </x:c>
       <x:c r="K92" s="12" t="str">
         <x:v>La Albiceleste</x:v>
       </x:c>
       <x:c r="L92" s="11" t="str">
-        <x:v>https://es.mlssoccer.com/noticias/messi-maradona-y-una-postal-bles-inolvidables-en-sunday-night-soccer</x:v>
+        <x:v>https://www.afa.com.ar/es/posts/125-goles-207-partidos-y-una-historia-que-cambio-para-siempre-a-la-seleccion-argentina</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="62" customHeight="1">
@@ -5312,7 +5312,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3490ad5579b4247"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2384871c8c4f423b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>